<commit_message>
wasn't accounting for fuel reserves needed for stage reuse
</commit_message>
<xml_diff>
--- a/launch_vehicle_design.xlsx
+++ b/launch_vehicle_design.xlsx
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M78"/>
+  <dimension ref="A1:M80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1073,89 +1073,95 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>LEO ΔV Fraction</t>
+          <t>Recovery ΔV Reserve (m/s)</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>0-1</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="n">
-        <v>0.597</v>
-      </c>
-      <c r="H23" s="9" t="n">
-        <v>0.403</v>
-      </c>
-      <c r="K23" s="9" t="inlineStr"/>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="H23" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>LEO ΔV Allocation</t>
+          <t>Recovery Propellant Reserved</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>m/s</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E24" s="14">
-        <f>IFERROR(E23*B37,"")</f>
+        <f>IFERROR(IF(E23=0,0,E58*(EXP(E23/(E28*9.80665))-1)),0)</f>
         <v/>
       </c>
       <c r="H24" s="14">
-        <f>IFERROR(H23*B37,"")</f>
+        <f>IFERROR(IF(H23=0,0,H58*(EXP(H23/(H28*9.80665))-1)),0)</f>
         <v/>
       </c>
       <c r="K24" s="14">
-        <f>IFERROR(K23*B37,"")</f>
+        <f>IFERROR(IF(K23=0,0,K58*(EXP(K23/(K28*9.80665))-1)),0)</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Vac Isp Override</t>
+          <t>LEO ΔV Fraction</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr"/>
-      <c r="H25" s="9" t="inlineStr"/>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="n">
+        <v>0.597</v>
+      </c>
+      <c r="H25" s="9" t="n">
+        <v>0.403</v>
+      </c>
       <c r="K25" s="9" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>Vac Isp (from DB)</t>
+          <t>LEO ΔV Allocation</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="E26" s="15">
-        <f>IF(E25&lt;&gt;"",E25,IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
-        <v/>
-      </c>
-      <c r="H26" s="15">
-        <f>IF(H25&lt;&gt;"",H25,IFERROR(VLOOKUP(H17,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
-        <v/>
-      </c>
-      <c r="K26" s="15">
-        <f>IF(K25&lt;&gt;"",K25,IFERROR(VLOOKUP(K17,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="E26" s="14">
+        <f>IFERROR(E25*B39,"")</f>
+        <v/>
+      </c>
+      <c r="H26" s="14">
+        <f>IFERROR(H25*B39,"")</f>
+        <v/>
+      </c>
+      <c r="K26" s="14">
+        <f>IFERROR(K25*B39,"")</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>SL Isp (from DB)</t>
+          <t>Vac Isp Override</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
@@ -1163,44 +1169,38 @@
           <t>s</t>
         </is>
       </c>
-      <c r="E27" s="15">
-        <f>IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,5,0),"—")</f>
-        <v/>
-      </c>
-      <c r="H27" s="15">
-        <f>IFERROR(VLOOKUP(H17,'Engine DB'!$A:$K,5,0),"—")</f>
-        <v/>
-      </c>
-      <c r="K27" s="15">
-        <f>IFERROR(VLOOKUP(K17,'Engine DB'!$A:$K,5,0),"—")</f>
-        <v/>
-      </c>
+      <c r="E27" s="9" t="inlineStr"/>
+      <c r="H27" s="9" t="inlineStr"/>
+      <c r="K27" s="9" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>Atm Fraction (0-1)</t>
+          <t>Vac Isp (from DB)</t>
         </is>
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H28" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="K28" s="9" t="n">
-        <v>1</v>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E28" s="15">
+        <f>IF(E27&lt;&gt;"",E27,IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+        <v/>
+      </c>
+      <c r="H28" s="15">
+        <f>IF(H27&lt;&gt;"",H27,IFERROR(VLOOKUP(H17,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+        <v/>
+      </c>
+      <c r="K28" s="15">
+        <f>IF(K27&lt;&gt;"",K27,IFERROR(VLOOKUP(K17,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Effective Isp (used)</t>
+          <t>SL Isp (from DB)</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
@@ -1208,222 +1208,219 @@
           <t>s</t>
         </is>
       </c>
-      <c r="E29" s="16">
-        <f>IFERROR(IF(ISNUMBER(E27),E27+E28*(E26-E27),E26),E26)</f>
-        <v/>
-      </c>
-      <c r="H29" s="16">
-        <f>IFERROR(IF(ISNUMBER(H27),H27+H28*(H26-H27),H26),H26)</f>
-        <v/>
-      </c>
-      <c r="K29" s="16">
-        <f>IFERROR(IF(ISNUMBER(K27),K27+K28*(K26-K27),K26),K26)</f>
+      <c r="E29" s="15">
+        <f>IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,5,0),"—")</f>
+        <v/>
+      </c>
+      <c r="H29" s="15">
+        <f>IFERROR(VLOOKUP(H17,'Engine DB'!$A:$K,5,0),"—")</f>
+        <v/>
+      </c>
+      <c r="K29" s="15">
+        <f>IFERROR(VLOOKUP(K17,'Engine DB'!$A:$K,5,0),"—")</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>GTO ΔV Fraction</t>
+          <t>Atm Fraction (0-1)</t>
         </is>
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E30" s="9" t="n">
-        <v>0.555</v>
+        <v>0.6</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>0.445</v>
-      </c>
-      <c r="K30" s="9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K30" s="9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
+          <t>Effective Isp (used)</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E31" s="16">
+        <f>IFERROR(IF(ISNUMBER(E29),E29+E30*(E28-E29),E28),E28)</f>
+        <v/>
+      </c>
+      <c r="H31" s="16">
+        <f>IFERROR(IF(ISNUMBER(H29),H29+H30*(H28-H29),H28),H28)</f>
+        <v/>
+      </c>
+      <c r="K31" s="16">
+        <f>IFERROR(IF(ISNUMBER(K29),K29+K30*(K28-K29),K28),K28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>GTO ΔV Fraction</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="n">
+        <v>0.555</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="K32" s="9" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
           <t>GTO ΔV Allocation</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
       </c>
-      <c r="E31" s="14">
-        <f>IFERROR(E30*B38,"")</f>
-        <v/>
-      </c>
-      <c r="H31" s="14">
-        <f>IFERROR(H30*B38,"")</f>
-        <v/>
-      </c>
-      <c r="K31" s="14">
-        <f>IFERROR(K30*B38,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="7" t="inlineStr">
+      <c r="E33" s="14">
+        <f>IFERROR(E32*B40,"")</f>
+        <v/>
+      </c>
+      <c r="H33" s="14">
+        <f>IFERROR(H32*B40,"")</f>
+        <v/>
+      </c>
+      <c r="K33" s="14">
+        <f>IFERROR(K32*B40,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>MISSION ΔV ANALYSIS  —  Gravity loss computed from liftoff TWR</t>
         </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
-        <is>
-          <t>Est. GLOW (stage masses only, no payload)</t>
-        </is>
-      </c>
-      <c r="B34" s="14">
-        <f>IFERROR(E20+E56,0)+IFERROR(H20+H56,0)+IFERROR(K20+K56,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>Stage 1 Liftoff TWR (est., no payload)</t>
-        </is>
-      </c>
-      <c r="B35" s="17">
-        <f>IFERROR(E18*IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,7,0),0)*1000/(B34*9.80665),"")</f>
-        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>Gravity Loss (= coeff / TWR)</t>
+          <t>Est. GLOW (stage masses only, no payload)</t>
         </is>
       </c>
       <c r="B36" s="14">
-        <f>IFERROR(B11/B35,"")</f>
+        <f>IFERROR(E20+E58,0)+IFERROR(H20+H58,0)+IFERROR(K20+K58,0)</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
         <is>
-          <t>LEO Mission ΔV (calculated)</t>
-        </is>
-      </c>
-      <c r="B37" s="18">
-        <f>IFERROR(B9+B10+B36,"")</f>
+          <t>Stage 1 Liftoff TWR (est., no payload)</t>
+        </is>
+      </c>
+      <c r="B37" s="17">
+        <f>IFERROR(E18*IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,7,0),0)*1000/(B36*9.80665),"")</f>
         <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>GTO Mission ΔV (calculated)</t>
-        </is>
-      </c>
-      <c r="B38" s="18">
-        <f>IFERROR(B12+B10+B36,"")</f>
+          <t>Gravity Loss (= coeff / TWR)</t>
+        </is>
+      </c>
+      <c r="B38" s="14">
+        <f>IFERROR(B11/B37,"")</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="19" t="inlineStr">
-        <is>
-          <t>LEO ΔV Allocation Check (should = LEO Mission ΔV above)</t>
-        </is>
-      </c>
-      <c r="B39" s="20">
-        <f>IFERROR(E24*1,0)+IFERROR(H24*1,0)+IFERROR(K24*1,0)</f>
-        <v/>
-      </c>
-      <c r="C39" s="2">
-        <f>IF(ABS(B39-B37)&lt;1,"✓ OK","⚠ Adjust stage allocations to sum to LEO Mission ΔV")</f>
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>LEO Mission ΔV (calculated)</t>
+        </is>
+      </c>
+      <c r="B39" s="18">
+        <f>IFERROR(B9+B10+B38,"")</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
+          <t>GTO Mission ΔV (calculated)</t>
+        </is>
+      </c>
+      <c r="B40" s="18">
+        <f>IFERROR(B12+B10+B38,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="19" t="inlineStr">
+        <is>
+          <t>LEO ΔV Allocation Check (should = LEO Mission ΔV above)</t>
+        </is>
+      </c>
+      <c r="B41" s="20">
+        <f>IFERROR(E26*1,0)+IFERROR(H26*1,0)+IFERROR(K26*1,0)</f>
+        <v/>
+      </c>
+      <c r="C41" s="2">
+        <f>IF(ABS(B41-B39)&lt;1,"✓ OK","⚠ Adjust stage allocations to sum to LEO Mission ΔV")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
           <t>Engine Mass per Engine</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E40" s="21">
+      <c r="E42" s="21">
         <f>IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,8,0),"—")</f>
         <v/>
       </c>
-      <c r="H40" s="21">
+      <c r="H42" s="21">
         <f>IFERROR(VLOOKUP(H17,'Engine DB'!$A:$K,8,0),"—")</f>
         <v/>
       </c>
-      <c r="K40" s="21">
+      <c r="K42" s="21">
         <f>IFERROR(VLOOKUP(K17,'Engine DB'!$A:$K,8,0),"—")</f>
         <v/>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="7" t="inlineStr">
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
         <is>
           <t>SUBSYSTEM MASS BREAKDOWN (auto-estimated; override any yellow cell)</t>
         </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="22" t="inlineStr">
-        <is>
-          <t>Tank Structure</t>
-        </is>
-      </c>
-      <c r="B43" s="12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E43" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",3.5,IF(E19="LOX/LH2",6.5,IF(E19="LOX/CH4",3.8,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),1.8,2.5)))))</f>
-        <v/>
-      </c>
-      <c r="H43" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",3.5,IF(H19="LOX/LH2",6.5,IF(H19="LOX/CH4",3.8,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),1.8,2.5)))))</f>
-        <v/>
-      </c>
-      <c r="K43" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",3.5,IF(K19="LOX/LH2",6.5,IF(K19="LOX/CH4",3.8,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),1.8,2.5)))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="22" t="inlineStr">
-        <is>
-          <t>Pressurization System</t>
-        </is>
-      </c>
-      <c r="B44" s="12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E44" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.4,IF(E19="LOX/LH2",0.6,IF(E19="LOX/CH4",0.4,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="H44" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.4,IF(H19="LOX/LH2",0.6,IF(H19="LOX/CH4",0.4,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="K44" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.4,IF(K19="LOX/LH2",0.6,IF(K19="LOX/CH4",0.4,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.0,0.5)))))</f>
-        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="22" t="inlineStr">
         <is>
-          <t>Feed System / Plumbing</t>
+          <t>Tank Structure</t>
         </is>
       </c>
       <c r="B45" s="12" t="inlineStr">
@@ -1432,22 +1429,22 @@
         </is>
       </c>
       <c r="E45" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.8,IF(E19="LOX/LH2",1.0,IF(E19="LOX/CH4",0.8,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.2,0.6)))))</f>
+        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",3.5,IF(E19="LOX/LH2",6.5,IF(E19="LOX/CH4",3.8,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),1.8,2.5)))))</f>
         <v/>
       </c>
       <c r="H45" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.8,IF(H19="LOX/LH2",1.0,IF(H19="LOX/CH4",0.8,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.2,0.6)))))</f>
+        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",3.5,IF(H19="LOX/LH2",6.5,IF(H19="LOX/CH4",3.8,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),1.8,2.5)))))</f>
         <v/>
       </c>
       <c r="K45" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.8,IF(K19="LOX/LH2",1.0,IF(K19="LOX/CH4",0.8,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.2,0.6)))))</f>
+        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",3.5,IF(K19="LOX/LH2",6.5,IF(K19="LOX/CH4",3.8,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),1.8,2.5)))))</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="22" t="inlineStr">
         <is>
-          <t>Avionics / GNC</t>
+          <t>Pressurization System</t>
         </is>
       </c>
       <c r="B46" s="12" t="inlineStr">
@@ -1456,22 +1453,22 @@
         </is>
       </c>
       <c r="E46" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.3,IF(E19="LOX/LH2",0.4,IF(E19="LOX/CH4",0.3,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.2,0.4)))))</f>
+        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.4,IF(E19="LOX/LH2",0.6,IF(E19="LOX/CH4",0.4,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.0,0.5)))))</f>
         <v/>
       </c>
       <c r="H46" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.3,IF(H19="LOX/LH2",0.4,IF(H19="LOX/CH4",0.3,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.2,0.4)))))</f>
+        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.4,IF(H19="LOX/LH2",0.6,IF(H19="LOX/CH4",0.4,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.0,0.5)))))</f>
         <v/>
       </c>
       <c r="K46" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.3,IF(K19="LOX/LH2",0.4,IF(K19="LOX/CH4",0.3,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.2,0.4)))))</f>
+        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.4,IF(K19="LOX/LH2",0.6,IF(K19="LOX/CH4",0.4,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.0,0.5)))))</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="22" t="inlineStr">
         <is>
-          <t>Power System</t>
+          <t>Feed System / Plumbing</t>
         </is>
       </c>
       <c r="B47" s="12" t="inlineStr">
@@ -1480,22 +1477,22 @@
         </is>
       </c>
       <c r="E47" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.2,IF(E19="LOX/LH2",0.3,IF(E19="LOX/CH4",0.2,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.8,IF(E19="LOX/LH2",1.0,IF(E19="LOX/CH4",0.8,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.2,0.6)))))</f>
         <v/>
       </c>
       <c r="H47" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.2,IF(H19="LOX/LH2",0.3,IF(H19="LOX/CH4",0.2,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.8,IF(H19="LOX/LH2",1.0,IF(H19="LOX/CH4",0.8,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.2,0.6)))))</f>
         <v/>
       </c>
       <c r="K47" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.2,IF(K19="LOX/LH2",0.3,IF(K19="LOX/CH4",0.2,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.8,IF(K19="LOX/LH2",1.0,IF(K19="LOX/CH4",0.8,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.2,0.6)))))</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="22" t="inlineStr">
         <is>
-          <t>Thermal Control</t>
+          <t>Avionics / GNC</t>
         </is>
       </c>
       <c r="B48" s="12" t="inlineStr">
@@ -1504,22 +1501,22 @@
         </is>
       </c>
       <c r="E48" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.2,IF(E19="LOX/LH2",1.0,IF(E19="LOX/CH4",0.3,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.1,0.3)))))</f>
+        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.3,IF(E19="LOX/LH2",0.4,IF(E19="LOX/CH4",0.3,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.2,0.4)))))</f>
         <v/>
       </c>
       <c r="H48" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.2,IF(H19="LOX/LH2",1.0,IF(H19="LOX/CH4",0.3,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.1,0.3)))))</f>
+        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.3,IF(H19="LOX/LH2",0.4,IF(H19="LOX/CH4",0.3,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.2,0.4)))))</f>
         <v/>
       </c>
       <c r="K48" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.2,IF(K19="LOX/LH2",1.0,IF(K19="LOX/CH4",0.3,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.1,0.3)))))</f>
+        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.3,IF(K19="LOX/LH2",0.4,IF(K19="LOX/CH4",0.3,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.2,0.4)))))</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="22" t="inlineStr">
         <is>
-          <t>RCS / ACS</t>
+          <t>Power System</t>
         </is>
       </c>
       <c r="B49" s="12" t="inlineStr">
@@ -1528,22 +1525,22 @@
         </is>
       </c>
       <c r="E49" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.3,IF(E19="LOX/LH2",0.4,IF(E19="LOX/CH4",0.3,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.2,IF(E19="LOX/LH2",0.3,IF(E19="LOX/CH4",0.2,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
       <c r="H49" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.3,IF(H19="LOX/LH2",0.4,IF(H19="LOX/CH4",0.3,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.2,IF(H19="LOX/LH2",0.3,IF(H19="LOX/CH4",0.2,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
       <c r="K49" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.3,IF(K19="LOX/LH2",0.4,IF(K19="LOX/CH4",0.3,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.2,IF(K19="LOX/LH2",0.3,IF(K19="LOX/CH4",0.2,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="22" t="inlineStr">
         <is>
-          <t>Separation System</t>
+          <t>Thermal Control</t>
         </is>
       </c>
       <c r="B50" s="12" t="inlineStr">
@@ -1552,22 +1549,22 @@
         </is>
       </c>
       <c r="E50" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.1,IF(E19="LOX/LH2",0.1,IF(E19="LOX/CH4",0.1,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.1,0.1)))))</f>
+        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.2,IF(E19="LOX/LH2",1.0,IF(E19="LOX/CH4",0.3,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.1,0.3)))))</f>
         <v/>
       </c>
       <c r="H50" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.1,IF(H19="LOX/LH2",0.1,IF(H19="LOX/CH4",0.1,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.1,0.1)))))</f>
+        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.2,IF(H19="LOX/LH2",1.0,IF(H19="LOX/CH4",0.3,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.1,0.3)))))</f>
         <v/>
       </c>
       <c r="K50" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.1,IF(K19="LOX/LH2",0.1,IF(K19="LOX/CH4",0.1,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.1,0.1)))))</f>
+        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.2,IF(K19="LOX/LH2",1.0,IF(K19="LOX/CH4",0.3,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.1,0.3)))))</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="22" t="inlineStr">
         <is>
-          <t>Recovery Hardware</t>
+          <t>RCS / ACS</t>
         </is>
       </c>
       <c r="B51" s="12" t="inlineStr">
@@ -1576,22 +1573,22 @@
         </is>
       </c>
       <c r="E51" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.0,IF(E19="LOX/LH2",0.0,IF(E19="LOX/CH4",0.0,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.0,0.0)))))</f>
+        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.3,IF(E19="LOX/LH2",0.4,IF(E19="LOX/CH4",0.3,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
       <c r="H51" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.0,IF(H19="LOX/LH2",0.0,IF(H19="LOX/CH4",0.0,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.0,0.0)))))</f>
+        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.3,IF(H19="LOX/LH2",0.4,IF(H19="LOX/CH4",0.3,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
       <c r="K51" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.0,IF(K19="LOX/LH2",0.0,IF(K19="LOX/CH4",0.0,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.0,0.0)))))</f>
+        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.3,IF(K19="LOX/LH2",0.4,IF(K19="LOX/CH4",0.3,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="22" t="inlineStr">
         <is>
-          <t>Residuals / Margin</t>
+          <t>Separation System</t>
         </is>
       </c>
       <c r="B52" s="12" t="inlineStr">
@@ -1600,203 +1597,203 @@
         </is>
       </c>
       <c r="E52" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.5,IF(E19="LOX/LH2",0.8,IF(E19="LOX/CH4",0.5,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.3,0.5)))))</f>
+        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.1,IF(E19="LOX/LH2",0.1,IF(E19="LOX/CH4",0.1,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.1,0.1)))))</f>
         <v/>
       </c>
       <c r="H52" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.5,IF(H19="LOX/LH2",0.8,IF(H19="LOX/CH4",0.5,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.3,0.5)))))</f>
+        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.1,IF(H19="LOX/LH2",0.1,IF(H19="LOX/CH4",0.1,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.1,0.1)))))</f>
         <v/>
       </c>
       <c r="K52" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.5,IF(K19="LOX/LH2",0.8,IF(K19="LOX/CH4",0.5,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.3,0.5)))))</f>
+        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.1,IF(K19="LOX/LH2",0.1,IF(K19="LOX/CH4",0.1,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.1,0.1)))))</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="22" t="inlineStr">
         <is>
+          <t>Recovery Hardware</t>
+        </is>
+      </c>
+      <c r="B53" s="12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E53" s="10">
+        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.0,IF(E19="LOX/LH2",0.0,IF(E19="LOX/CH4",0.0,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.0,0.0)))))</f>
+        <v/>
+      </c>
+      <c r="H53" s="10">
+        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.0,IF(H19="LOX/LH2",0.0,IF(H19="LOX/CH4",0.0,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.0,0.0)))))</f>
+        <v/>
+      </c>
+      <c r="K53" s="10">
+        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.0,IF(K19="LOX/LH2",0.0,IF(K19="LOX/CH4",0.0,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.0,0.0)))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="22" t="inlineStr">
+        <is>
+          <t>Residuals / Margin</t>
+        </is>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E54" s="10">
+        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.5,IF(E19="LOX/LH2",0.8,IF(E19="LOX/CH4",0.5,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.3,0.5)))))</f>
+        <v/>
+      </c>
+      <c r="H54" s="10">
+        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.5,IF(H19="LOX/LH2",0.8,IF(H19="LOX/CH4",0.5,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.3,0.5)))))</f>
+        <v/>
+      </c>
+      <c r="K54" s="10">
+        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.5,IF(K19="LOX/LH2",0.8,IF(K19="LOX/CH4",0.5,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.3,0.5)))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="22" t="inlineStr">
+        <is>
           <t>Engine System Total</t>
         </is>
       </c>
-      <c r="B53" s="12" t="inlineStr">
+      <c r="B55" s="12" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E53" s="21">
-        <f>IFERROR(E18*E40*1.15, "")</f>
-        <v/>
-      </c>
-      <c r="H53" s="21">
-        <f>IFERROR(H18*H40*1.15, "")</f>
-        <v/>
-      </c>
-      <c r="K53" s="21">
-        <f>IFERROR(K18*K40*1.15, "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="23" t="inlineStr">
+      <c r="E55" s="21">
+        <f>IFERROR(E18*E42*1.15, "")</f>
+        <v/>
+      </c>
+      <c r="H55" s="21">
+        <f>IFERROR(H18*H42*1.15, "")</f>
+        <v/>
+      </c>
+      <c r="K55" s="21">
+        <f>IFERROR(K18*K42*1.15, "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="23" t="inlineStr">
         <is>
           <t>TOTAL DRY MASS (Estimated)</t>
         </is>
       </c>
-      <c r="B54" s="24" t="inlineStr">
+      <c r="B56" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E54" s="13">
-        <f>IFERROR(E43+E44+E45+E46+E47+E48+E49+E50+E51+E52+E53, "")</f>
-        <v/>
-      </c>
-      <c r="H54" s="13">
-        <f>IFERROR(H43+H44+H45+H46+H47+H48+H49+H50+H51+H52+H53, "")</f>
-        <v/>
-      </c>
-      <c r="K54" s="13">
-        <f>IFERROR(K43+K44+K45+K46+K47+K48+K49+K50+K51+K52+K53, "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="8" t="inlineStr">
+      <c r="E56" s="13">
+        <f>IFERROR(E45+E46+E47+E48+E49+E50+E51+E52+E53+E54+E55, "")</f>
+        <v/>
+      </c>
+      <c r="H56" s="13">
+        <f>IFERROR(H45+H46+H47+H48+H49+H50+H51+H52+H53+H54+H55, "")</f>
+        <v/>
+      </c>
+      <c r="K56" s="13">
+        <f>IFERROR(K45+K46+K47+K48+K49+K50+K51+K52+K53+K54+K55, "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="inlineStr">
         <is>
           <t>Dry Mass Override (enter known value)</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B57" s="12" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E55" s="10" t="inlineStr"/>
-      <c r="H55" s="10" t="inlineStr"/>
-      <c r="K55" s="10" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="inlineStr">
+      <c r="E57" s="10" t="inlineStr"/>
+      <c r="H57" s="10" t="inlineStr"/>
+      <c r="K57" s="10" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
         <is>
           <t>Effective Dry Mass</t>
         </is>
       </c>
-      <c r="B56" s="12" t="inlineStr">
+      <c r="B58" s="12" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E56" s="21">
-        <f>IF(E55&lt;&gt;"",E55,E54)</f>
-        <v/>
-      </c>
-      <c r="H56" s="21">
-        <f>IF(H55&lt;&gt;"",H55,H54)</f>
-        <v/>
-      </c>
-      <c r="K56" s="21">
-        <f>IF(K55&lt;&gt;"",K55,K54)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="7" t="inlineStr">
+      <c r="E58" s="21">
+        <f>IF(E57&lt;&gt;"",E57,E56)</f>
+        <v/>
+      </c>
+      <c r="H58" s="21">
+        <f>IF(H57&lt;&gt;"",H57,H56)</f>
+        <v/>
+      </c>
+      <c r="K58" s="21">
+        <f>IF(K57&lt;&gt;"",K57,K56)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>PERFORMANCE CALCULATIONS</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="25" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="25" t="inlineStr">
         <is>
           <t>MAX PAYLOAD TO ORBIT</t>
         </is>
       </c>
-      <c r="B59" s="26">
-        <f>IF(B13&gt;=3,IFERROR(K22/(EXP(K24/(K29*9.80665))-1)-K56-B8, ""),IF(B13&gt;=2,IFERROR(H22/(EXP(H24/(H29*9.80665))-1)-H56-B8, ""),IFERROR(E22/(EXP(E24/(E29*9.80665))-1)-E56-B8, "")))</f>
-        <v/>
-      </c>
-      <c r="C59" s="27" t="inlineStr">
-        <is>
-          <t>← Solved from last stage: m_payload = prop/(e^(ΔV/Isp·g₀)−1) − dry − adapter</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="7" t="inlineStr">
+      <c r="B61" s="26">
+        <f>IF(B13&gt;=3,IFERROR((K22-K24)/(EXP(K26/(K31*9.80665))-1)-(K58+K24)-B8, ""),IF(B13&gt;=2,IFERROR((H22-H24)/(EXP(H26/(H31*9.80665))-1)-(H58+H24)-B8, ""),IFERROR((E22-E24)/(EXP(E26/(E31*9.80665))-1)-(E58+E24)-B8, "")))</f>
+        <v/>
+      </c>
+      <c r="C61" s="27" t="inlineStr">
+        <is>
+          <t>← Solved from last stage: m_payload = (prop−rec)/(e^(ΔV/Isp·g₀)−1) − (dry+rec) − adapter  |  Recovery penalty: lower stage's actual ΔV drops (see verification); reduce that stage's ΔV fraction to propagate penalty to payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="7" t="inlineStr">
         <is>
           <t>GTO PERFORMANCE</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="25" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="25" t="inlineStr">
         <is>
           <t>MAX PAYLOAD TO GTO</t>
         </is>
       </c>
-      <c r="B62" s="26">
-        <f>IF(B13&gt;=3,IFERROR(K22/(EXP(K31/(K29*9.80665))-1)-K56-B8, ""),IF(B13&gt;=2,IFERROR(H22/(EXP(H31/(H29*9.80665))-1)-H56-B8, ""),IFERROR(E22/(EXP(E31/(E29*9.80665))-1)-E56-B8, "")))</f>
-        <v/>
-      </c>
-      <c r="C62" s="27" t="inlineStr">
-        <is>
-          <t>← Solved from last stage using GTO ΔV allocations: m_payload = prop/(e^(ΔV/Isp·g₀)−1) − dry − adapter</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="8" t="inlineStr">
-        <is>
-          <t>Gross Stage Mass (Prop + Dry)</t>
-        </is>
-      </c>
-      <c r="B63" s="12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E63" s="21">
-        <f>IFERROR(E22+E56, "")</f>
-        <v/>
-      </c>
-      <c r="H63" s="21">
-        <f>IFERROR(H22+H56, "")</f>
-        <v/>
-      </c>
-      <c r="K63" s="21">
-        <f>IFERROR(K22+K56, "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="8" t="inlineStr">
-        <is>
-          <t>Burnout Mass m_f</t>
-        </is>
-      </c>
-      <c r="B64" s="12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E64" s="21">
-        <f>IFERROR(E56+IFERROR(H63*1,0)+IFERROR(K63*1,0)+B59+B8, "")</f>
-        <v/>
-      </c>
-      <c r="H64" s="21">
-        <f>IFERROR(H56+IFERROR(K63*1,0)+B59+B8, "")</f>
-        <v/>
-      </c>
-      <c r="K64" s="21">
-        <f>IFERROR(K56+B59+B8, "")</f>
-        <v/>
+      <c r="B64" s="26">
+        <f>IF(B13&gt;=3,IFERROR((K22-K24)/(EXP(K33/(K31*9.80665))-1)-(K58+K24)-B8, ""),IF(B13&gt;=2,IFERROR((H22-H24)/(EXP(H33/(H31*9.80665))-1)-(H58+H24)-B8, ""),IFERROR((E22-E24)/(EXP(E33/(E31*9.80665))-1)-(E58+E24)-B8, "")))</f>
+        <v/>
+      </c>
+      <c r="C64" s="27" t="inlineStr">
+        <is>
+          <t>← MIN across all stage constraints using GTO ΔV allocations: capacity_i = (prop−rec)/(e^(ΔV/Isp·g₀)−1) − (dry+rec) − gross_above − adapter</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>Initial Mass m_0 (at ignition)</t>
+          <t>Gross Stage Mass (Prop + Dry)</t>
         </is>
       </c>
       <c r="B65" s="12" t="inlineStr">
@@ -1805,228 +1802,276 @@
         </is>
       </c>
       <c r="E65" s="21">
-        <f>IFERROR(E64+E22, "")</f>
+        <f>IFERROR(E22+E58, "")</f>
         <v/>
       </c>
       <c r="H65" s="21">
-        <f>IFERROR(H64+H22, "")</f>
+        <f>IFERROR(H22+H58, "")</f>
         <v/>
       </c>
       <c r="K65" s="21">
-        <f>IFERROR(K64+K22, "")</f>
+        <f>IFERROR(K22+K58, "")</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>Mass Ratio (m₀ / m_f)</t>
+          <t>Burnout Mass m_f</t>
         </is>
       </c>
       <c r="B66" s="12" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E66" s="28">
-        <f>IFERROR(E65/E64, "")</f>
-        <v/>
-      </c>
-      <c r="H66" s="28">
-        <f>IFERROR(H65/H64, "")</f>
-        <v/>
-      </c>
-      <c r="K66" s="28">
-        <f>IFERROR(K65/K64, "")</f>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E66" s="21">
+        <f>IFERROR(E58+E24+IFERROR(H65*1,0)+IFERROR(K65*1,0)+B61+B8, "")</f>
+        <v/>
+      </c>
+      <c r="H66" s="21">
+        <f>IFERROR(H58+H24+IFERROR(K65*1,0)+B61+B8, "")</f>
+        <v/>
+      </c>
+      <c r="K66" s="21">
+        <f>IFERROR(K58+K24+B61+B8, "")</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="23" t="inlineStr">
-        <is>
-          <t>Actual Stage ΔV (verification)</t>
-        </is>
-      </c>
-      <c r="B67" s="24" t="inlineStr">
-        <is>
-          <t>m/s</t>
-        </is>
-      </c>
-      <c r="E67" s="13">
-        <f>IFERROR(E29*9.80665*LN(E66), "")</f>
-        <v/>
-      </c>
-      <c r="H67" s="13">
-        <f>IFERROR(H29*9.80665*LN(H66), "")</f>
-        <v/>
-      </c>
-      <c r="K67" s="13">
-        <f>IFERROR(K29*9.80665*LN(K66), "")</f>
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>Initial Mass m_0 (at ignition)</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E67" s="21">
+        <f>IFERROR(E66+E22-E24, "")</f>
+        <v/>
+      </c>
+      <c r="H67" s="21">
+        <f>IFERROR(H66+H22-H24, "")</f>
+        <v/>
+      </c>
+      <c r="K67" s="21">
+        <f>IFERROR(K66+K22-K24, "")</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
+          <t>Mass Ratio (m₀ / m_f)</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E68" s="28">
+        <f>IFERROR(E67/E66, "")</f>
+        <v/>
+      </c>
+      <c r="H68" s="28">
+        <f>IFERROR(H67/H66, "")</f>
+        <v/>
+      </c>
+      <c r="K68" s="28">
+        <f>IFERROR(K67/K66, "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="23" t="inlineStr">
+        <is>
+          <t>Actual Stage ΔV (verification)</t>
+        </is>
+      </c>
+      <c r="B69" s="24" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="E69" s="13">
+        <f>IFERROR(E31*9.80665*LN(E68), "")</f>
+        <v/>
+      </c>
+      <c r="H69" s="13">
+        <f>IFERROR(H31*9.80665*LN(H68), "")</f>
+        <v/>
+      </c>
+      <c r="K69" s="13">
+        <f>IFERROR(K31*9.80665*LN(K68), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="8" t="inlineStr">
+        <is>
           <t>Thrust-to-Weight Ratio (at ignition)</t>
         </is>
       </c>
-      <c r="B68" s="12" t="inlineStr">
+      <c r="B70" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E68" s="29">
-        <f>IFERROR(E18*IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,7,0),0)*1000/(E65*9.80665), "")</f>
-        <v/>
-      </c>
-      <c r="H68" s="29">
-        <f>IFERROR(H18*IFERROR(VLOOKUP(H17,'Engine DB'!$A:$K,6,0),0)*1000/(H65*9.80665), "")</f>
-        <v/>
-      </c>
-      <c r="K68" s="29">
-        <f>IFERROR(K18*IFERROR(VLOOKUP(K17,'Engine DB'!$A:$K,6,0),0)*1000/(K65*9.80665), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="8" t="inlineStr">
+      <c r="E70" s="29">
+        <f>IFERROR(E18*IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,7,0),0)*1000/(E67*9.80665), "")</f>
+        <v/>
+      </c>
+      <c r="H70" s="29">
+        <f>IFERROR(H18*IFERROR(VLOOKUP(H17,'Engine DB'!$A:$K,6,0),0)*1000/(H67*9.80665), "")</f>
+        <v/>
+      </c>
+      <c r="K70" s="29">
+        <f>IFERROR(K18*IFERROR(VLOOKUP(K17,'Engine DB'!$A:$K,6,0),0)*1000/(K67*9.80665), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
         <is>
           <t>Propellant Mass Fraction</t>
         </is>
       </c>
-      <c r="B69" s="12" t="inlineStr">
+      <c r="B71" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E69" s="28">
-        <f>IFERROR(E22/E65, "")</f>
-        <v/>
-      </c>
-      <c r="H69" s="28">
-        <f>IFERROR(H22/H65, "")</f>
-        <v/>
-      </c>
-      <c r="K69" s="28">
-        <f>IFERROR(K22/K65, "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="71" ht="18" customHeight="1">
-      <c r="A71" s="7" t="inlineStr">
+      <c r="E71" s="28">
+        <f>IFERROR(E22/E67, "")</f>
+        <v/>
+      </c>
+      <c r="H71" s="28">
+        <f>IFERROR(H22/H67, "")</f>
+        <v/>
+      </c>
+      <c r="K71" s="28">
+        <f>IFERROR(K22/K67, "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="7" t="inlineStr">
         <is>
           <t>VEHICLE SUMMARY</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="30" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="30" t="inlineStr">
         <is>
           <t>Max Payload to LEO</t>
         </is>
       </c>
-      <c r="B72" s="31">
-        <f>B59</f>
-        <v/>
-      </c>
-      <c r="C72" s="32" t="inlineStr">
+      <c r="B74" s="31">
+        <f>B61</f>
+        <v/>
+      </c>
+      <c r="C74" s="32" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="30" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="30" t="inlineStr">
         <is>
           <t>Max Payload to GTO</t>
         </is>
       </c>
-      <c r="B73" s="31">
-        <f>B62</f>
-        <v/>
-      </c>
-      <c r="C73" s="32" t="inlineStr">
+      <c r="B75" s="31">
+        <f>B64</f>
+        <v/>
+      </c>
+      <c r="C75" s="32" t="inlineStr">
         <is>
           <t>kg</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="33" t="inlineStr">
-        <is>
-          <t>LEO Payload Fraction (GLOW)</t>
-        </is>
-      </c>
-      <c r="B74" s="34">
-        <f>IFERROR(B59/E65*100, "")</f>
-        <v/>
-      </c>
-      <c r="C74" s="32" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="33" t="inlineStr">
-        <is>
-          <t>Total Vehicle ΔV (actual)</t>
-        </is>
-      </c>
-      <c r="B75" s="35">
-        <f>IFERROR(E67*1,0)+IFERROR(H67*1,0)+IFERROR(K67*1,0)</f>
-        <v/>
-      </c>
-      <c r="C75" s="32" t="inlineStr">
-        <is>
-          <t>m/s</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="33" t="inlineStr">
         <is>
-          <t>LEO ΔV Margin vs Mission</t>
-        </is>
-      </c>
-      <c r="B76" s="35">
-        <f>IFERROR(E67*1,0)+IFERROR(H67*1,0)+IFERROR(K67*1,0)-B37</f>
+          <t>LEO Payload Fraction (GLOW)</t>
+        </is>
+      </c>
+      <c r="B76" s="34">
+        <f>IFERROR(B61/E67*100, "")</f>
         <v/>
       </c>
       <c r="C76" s="32" t="inlineStr">
         <is>
-          <t>m/s</t>
+          <t>%</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="33" t="inlineStr">
         <is>
-          <t>Gross Liftoff Mass (GLOW)</t>
+          <t>Total Vehicle ΔV (actual)</t>
         </is>
       </c>
       <c r="B77" s="35">
-        <f>IFERROR(E65, "")</f>
+        <f>IFERROR(E69*1,0)+IFERROR(H69*1,0)+IFERROR(K69*1,0)</f>
         <v/>
       </c>
       <c r="C77" s="32" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m/s</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="33" t="inlineStr">
         <is>
+          <t>LEO ΔV Margin vs Mission</t>
+        </is>
+      </c>
+      <c r="B78" s="35">
+        <f>IFERROR(E69*1,0)+IFERROR(H69*1,0)+IFERROR(K69*1,0)-B39</f>
+        <v/>
+      </c>
+      <c r="C78" s="32" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="33" t="inlineStr">
+        <is>
+          <t>Gross Liftoff Mass (GLOW)</t>
+        </is>
+      </c>
+      <c r="B79" s="35">
+        <f>IFERROR(E67, "")</f>
+        <v/>
+      </c>
+      <c r="C79" s="32" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="33" t="inlineStr">
+        <is>
           <t>Total Propellant Mass</t>
         </is>
       </c>
-      <c r="B78" s="35">
+      <c r="B80" s="35">
         <f>IFERROR(E22,0)+IFERROR(H22,0)+IFERROR(K22,0)</f>
         <v/>
       </c>
-      <c r="C78" s="32" t="inlineStr">
+      <c r="C80" s="32" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -2034,25 +2079,25 @@
     </row>
   </sheetData>
   <mergeCells count="21">
-    <mergeCell ref="A58:K58"/>
-    <mergeCell ref="C39:L39"/>
+    <mergeCell ref="C61:L61"/>
     <mergeCell ref="C8:L8"/>
     <mergeCell ref="A15:K15"/>
-    <mergeCell ref="A61:K61"/>
+    <mergeCell ref="A73:K73"/>
+    <mergeCell ref="A60:K60"/>
     <mergeCell ref="C13:L13"/>
-    <mergeCell ref="C62:L62"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="A1:M1"/>
+    <mergeCell ref="C64:L64"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A33:K33"/>
-    <mergeCell ref="A71:K71"/>
-    <mergeCell ref="A42:K42"/>
     <mergeCell ref="C10:L10"/>
     <mergeCell ref="D3:E3"/>
+    <mergeCell ref="C41:L41"/>
     <mergeCell ref="J3:K3"/>
+    <mergeCell ref="A35:K35"/>
     <mergeCell ref="C9:L9"/>
-    <mergeCell ref="C59:L59"/>
+    <mergeCell ref="A63:K63"/>
     <mergeCell ref="C12:L12"/>
+    <mergeCell ref="A44:K44"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="C11:L11"/>
   </mergeCells>
@@ -2067,7 +2112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2173,182 +2218,248 @@
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="37" t="inlineStr">
         <is>
-          <t>5.  Performance section calculates automatically:</t>
+          <t>5.  For reusable stages (e.g. New Glenn S1, Falcon 9 S1), enter a Recovery ΔV Reserve:</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">      • Delta-V per stage via Tsiolkovsky equation: ΔV = Isp × g₀ × ln(m₀/m_f)</t>
+          <t xml:space="preserve">      • This is the total ΔV budget for recovery burns (boost-back + entry + landing).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">      • Burnout mass accounts for all upper stages + payload + payload adapter.</t>
+          <t xml:space="preserve">      • Typical values: ~750 m/s for RTLS (return-to-launch-site), ~500 m/s for ASDS (drone ship).</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">      • TWR uses sea-level thrust for Stage 1, vacuum thrust for upper stages.</t>
+          <t xml:space="preserve">      • The tool computes Recovery Propellant Reserved = dry_mass × (e^(ΔV/Isp/g₀) − 1).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="37" t="inlineStr"/>
+      <c r="A21" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      • This propellant is treated as dead weight during ascent (still onboard at MECO).</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="36" t="inlineStr">
-        <is>
-          <t>TIPS &amp; RULES OF THUMB</t>
+      <c r="A22" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      • Set to 0 for expendable stages — no penalty applied.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="37" t="inlineStr">
-        <is>
-          <t>• LEO missions typically need 9,000–9,500 m/s total ΔV (includes ~1,500 m/s gravity+drag losses).</t>
-        </is>
-      </c>
+      <c r="A23" s="37" t="inlineStr"/>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="37" t="inlineStr">
         <is>
-          <t>• GTO missions need ~11,500–12,500 m/s depending on inclination.</t>
+          <t>6.  Performance section calculates automatically:</t>
         </is>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="37" t="inlineStr">
         <is>
-          <t>• First stage TWR should be 1.2–1.5 at liftoff; too low = slow ascent; too high = unnecessary mass.</t>
+          <t xml:space="preserve">      • Delta-V per stage via Tsiolkovsky equation: ΔV = Isp × g₀ × ln(m₀/m_f)</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="37" t="inlineStr">
         <is>
-          <t>• Payload fraction for real vehicles: 1.5–4% to LEO is typical.</t>
+          <t xml:space="preserve">      • Burnout mass includes recovery-reserved propellant (still onboard at MECO) for reusable stages.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="37" t="inlineStr">
         <is>
-          <t>• Structural mass fraction (dry/propellant) is typically 5–15%; lower is better engineering.</t>
+          <t xml:space="preserve">      • TWR uses sea-level thrust for Stage 1, vacuum thrust for upper stages.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="37" t="inlineStr">
-        <is>
-          <t>• LOX/LH2 gives the highest Isp (~450s) but low density means large, heavy tanks.</t>
-        </is>
-      </c>
+      <c r="A28" s="37" t="inlineStr"/>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="37" t="inlineStr">
-        <is>
-          <t>• LOX/RP-1 gives good density and SL performance; workhorse of most first stages.</t>
+      <c r="A29" s="36" t="inlineStr">
+        <is>
+          <t>TIPS &amp; RULES OF THUMB</t>
         </is>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="37" t="inlineStr">
         <is>
-          <t>• LOX/CH4 is the emerging choice for reusability; good Isp + density balance.</t>
+          <t>• LEO missions typically need 9,000–9,500 m/s total ΔV (includes ~1,500 m/s gravity+drag losses).</t>
         </is>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="37" t="inlineStr"/>
+      <c r="A31" s="37" t="inlineStr">
+        <is>
+          <t>• GTO missions need ~11,500–12,500 m/s depending on inclination.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="36" t="inlineStr">
-        <is>
-          <t>REFERENCE TABS</t>
+      <c r="A32" s="37" t="inlineStr">
+        <is>
+          <t>• First stage TWR should be 1.2–1.5 at liftoff; too low = slow ascent; too high = unnecessary mass.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="37" t="inlineStr">
         <is>
-          <t>• Engine DB:   Real engine performance data for 35+ engines. Add your own rows at the bottom.</t>
+          <t>• Payload fraction for real vehicles: 1.5–4% to LEO is typical.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="37" t="inlineStr">
         <is>
-          <t>• Vehicle DB:  Real vehicle mass breakdowns for 11 vehicles. Use for design grounding.</t>
+          <t>• Structural mass fraction (dry/propellant) is typically 5–15%; lower is better engineering.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="37" t="inlineStr">
         <is>
-          <t>• Propellants: Propellant properties + subsystem mass fraction model documentation.</t>
+          <t>• LOX/LH2 gives the highest Isp (~450s) but low density means large, heavy tanks.</t>
         </is>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="37" t="inlineStr">
         <is>
-          <t>• Comparison:  Quick performance comparison table across all reference vehicles.</t>
+          <t>• LOX/RP-1 gives good density and SL performance; workhorse of most first stages.</t>
         </is>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="37" t="inlineStr"/>
+      <c r="A37" s="37" t="inlineStr">
+        <is>
+          <t>• LOX/CH4 is the emerging choice for reusability; good Isp + density balance.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="36" t="inlineStr">
-        <is>
-          <t>LIMITATIONS</t>
+      <c r="A38" s="37" t="inlineStr">
+        <is>
+          <t>• Reusable first stages carry a payload penalty: ~30–40% less to LEO vs expendable (Falcon 9 example).</t>
         </is>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="37" t="inlineStr">
         <is>
-          <t>• This tool uses simplified mass models. Real designs require detailed MDO and stress analysis.</t>
+          <t>• Recovery ΔV budget: RTLS ~750 m/s (boost-back ~300 + entry ~200 + landing ~250);</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="37" t="inlineStr">
         <is>
-          <t>• Delta-V calculations assume impulsive burns (no trajectory shaping or staging timing).</t>
+          <t xml:space="preserve">  ASDS (drone ship) ~450–500 m/s (no boost-back; entry ~200 + landing ~250).</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="37" t="inlineStr">
-        <is>
-          <t>• Subsystem fractions are statistical — early concept accuracy is ±20–30%.</t>
-        </is>
-      </c>
+      <c r="A41" s="37" t="inlineStr"/>
     </row>
     <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="37" t="inlineStr">
-        <is>
-          <t>• Solid stages show N/A for SL Isp in engine DB — use Vac Isp as a conservative estimate.</t>
+      <c r="A42" s="36" t="inlineStr">
+        <is>
+          <t>REFERENCE TABS</t>
         </is>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="37" t="inlineStr">
         <is>
-          <t>• Parallel staging (e.g. strap-on boosters firing simultaneously with a core) is not modeled.</t>
+          <t>• Engine DB:   Real engine performance data for 35+ engines. Add your own rows at the bottom.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="37" t="inlineStr">
+        <is>
+          <t>• Vehicle DB:  Real vehicle mass breakdowns for 11 vehicles. Use for design grounding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="37" t="inlineStr">
+        <is>
+          <t>• Propellants: Propellant properties + subsystem mass fraction model documentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="37" t="inlineStr">
+        <is>
+          <t>• Comparison:  Quick performance comparison table across all reference vehicles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="16" customHeight="1">
+      <c r="A47" s="37" t="inlineStr"/>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="A48" s="36" t="inlineStr">
+        <is>
+          <t>LIMITATIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="37" t="inlineStr">
+        <is>
+          <t>• This tool uses simplified mass models. Real designs require detailed MDO and stress analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="16" customHeight="1">
+      <c r="A50" s="37" t="inlineStr">
+        <is>
+          <t>• Delta-V calculations assume impulsive burns (no trajectory shaping or staging timing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="16" customHeight="1">
+      <c r="A51" s="37" t="inlineStr">
+        <is>
+          <t>• Subsystem fractions are statistical — early concept accuracy is ±20–30%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="37" t="inlineStr">
+        <is>
+          <t>• Solid stages show N/A for SL Isp in engine DB — use Vac Isp as a conservative estimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="37" t="inlineStr">
+        <is>
+          <t>• Parallel staging (e.g. strap-on boosters firing simultaneously with a core) is not modeled.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">  Treat parallel-burn vehicles (Soyuz, Ariane 5) as series stages for delta-v calculation.</t>
         </is>
@@ -2366,7 +2477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -3674,263 +3785,263 @@
       </c>
       <c r="K32" s="39" t="inlineStr">
         <is>
-          <t>Upgraded BE-4; 2,847 kN SL (640,000 lbf) with propellant subcooling; vac est. proportional; same Isp</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="7" t="inlineStr">
+          <t>Upgraded BE-4 with subcooling; 2,847 kN SL (640,000 lbf); use with Subcooling Gain ~3.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" s="39" t="inlineStr">
+        <is>
+          <t>BE-4 Block 2 (no subcool)</t>
+        </is>
+      </c>
+      <c r="B33" s="39" t="inlineStr">
+        <is>
+          <t>New Glenn Block 2 S1</t>
+        </is>
+      </c>
+      <c r="C33" s="40" t="inlineStr">
+        <is>
+          <t>LOX/CH4</t>
+        </is>
+      </c>
+      <c r="D33" s="40" t="n">
+        <v>339</v>
+      </c>
+      <c r="E33" s="40" t="n">
+        <v>310</v>
+      </c>
+      <c r="F33" s="40" t="n">
+        <v>2780</v>
+      </c>
+      <c r="G33" s="40" t="n">
+        <v>2430</v>
+      </c>
+      <c r="H33" s="40" t="n">
+        <v>4760</v>
+      </c>
+      <c r="I33" s="40" t="n">
+        <v>134</v>
+      </c>
+      <c r="J33" s="40" t="n">
+        <v>40</v>
+      </c>
+      <c r="K33" s="39" t="inlineStr">
+        <is>
+          <t>Upgraded BE-4 design improvements only, no subcooling; 2,780 kN SL (625,000 lbf); use with Subcooling Gain 0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>── NTO/MMH ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="15" customHeight="1">
-      <c r="A34" s="39" t="inlineStr">
-        <is>
-          <t>AJ-10-190</t>
-        </is>
-      </c>
-      <c r="B34" s="39" t="inlineStr">
-        <is>
-          <t>Orion SPS / STS OMS</t>
-        </is>
-      </c>
-      <c r="C34" s="40" t="inlineStr">
-        <is>
-          <t>NTO/MMH</t>
-        </is>
-      </c>
-      <c r="D34" s="40" t="n">
-        <v>316</v>
-      </c>
-      <c r="E34" s="40" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F34" s="40" t="n">
-        <v>27</v>
-      </c>
-      <c r="G34" s="40" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H34" s="40" t="n">
-        <v>118</v>
-      </c>
-      <c r="I34" s="40" t="n">
-        <v>9</v>
-      </c>
-      <c r="J34" s="40" t="n">
-        <v>49</v>
-      </c>
-      <c r="K34" s="39" t="inlineStr">
-        <is>
-          <t>Pressure-fed; restartable; long heritage</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="39" t="inlineStr">
         <is>
+          <t>AJ-10-190</t>
+        </is>
+      </c>
+      <c r="B35" s="39" t="inlineStr">
+        <is>
+          <t>Orion SPS / STS OMS</t>
+        </is>
+      </c>
+      <c r="C35" s="40" t="inlineStr">
+        <is>
+          <t>NTO/MMH</t>
+        </is>
+      </c>
+      <c r="D35" s="40" t="n">
+        <v>316</v>
+      </c>
+      <c r="E35" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F35" s="40" t="n">
+        <v>27</v>
+      </c>
+      <c r="G35" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="40" t="n">
+        <v>118</v>
+      </c>
+      <c r="I35" s="40" t="n">
+        <v>9</v>
+      </c>
+      <c r="J35" s="40" t="n">
+        <v>49</v>
+      </c>
+      <c r="K35" s="39" t="inlineStr">
+        <is>
+          <t>Pressure-fed; restartable; long heritage</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="15" customHeight="1">
+      <c r="A36" s="39" t="inlineStr">
+        <is>
           <t>Aestus</t>
         </is>
       </c>
-      <c r="B35" s="39" t="inlineStr">
+      <c r="B36" s="39" t="inlineStr">
         <is>
           <t>Ariane 5 ATV</t>
         </is>
       </c>
-      <c r="C35" s="40" t="inlineStr">
+      <c r="C36" s="40" t="inlineStr">
         <is>
           <t>NTO/MMH</t>
         </is>
       </c>
-      <c r="D35" s="40" t="n">
+      <c r="D36" s="40" t="n">
         <v>324</v>
       </c>
-      <c r="E35" s="40" t="inlineStr">
+      <c r="E36" s="40" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F35" s="40" t="n">
+      <c r="F36" s="40" t="n">
         <v>29</v>
       </c>
-      <c r="G35" s="40" t="inlineStr">
+      <c r="G36" s="40" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H35" s="40" t="n">
+      <c r="H36" s="40" t="n">
         <v>111</v>
       </c>
-      <c r="I35" s="40" t="n">
+      <c r="I36" s="40" t="n">
         <v>11</v>
       </c>
-      <c r="J35" s="40" t="n">
+      <c r="J36" s="40" t="n">
         <v>84</v>
       </c>
-      <c r="K35" s="39" t="inlineStr">
+      <c r="K36" s="39" t="inlineStr">
         <is>
           <t>Pressure-fed; restartable; ESA upper stage</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="7" t="inlineStr">
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>── NTO/UDMH ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="39" t="inlineStr">
-        <is>
-          <t>Vikas</t>
-        </is>
-      </c>
-      <c r="B37" s="39" t="inlineStr">
-        <is>
-          <t>PSLV / GSLV S2</t>
-        </is>
-      </c>
-      <c r="C37" s="40" t="inlineStr">
-        <is>
-          <t>NTO/UDMH</t>
-        </is>
-      </c>
-      <c r="D37" s="40" t="n">
-        <v>293</v>
-      </c>
-      <c r="E37" s="40" t="n">
-        <v>270</v>
-      </c>
-      <c r="F37" s="40" t="n">
-        <v>800</v>
-      </c>
-      <c r="G37" s="40" t="n">
-        <v>725</v>
-      </c>
-      <c r="H37" s="40" t="n">
-        <v>634</v>
-      </c>
-      <c r="I37" s="40" t="n">
-        <v>58</v>
-      </c>
-      <c r="J37" s="40" t="n">
-        <v>16</v>
-      </c>
-      <c r="K37" s="39" t="inlineStr">
-        <is>
-          <t>Indian engine; Ariane Viking derivative</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="39" t="inlineStr">
         <is>
+          <t>Vikas</t>
+        </is>
+      </c>
+      <c r="B38" s="39" t="inlineStr">
+        <is>
+          <t>PSLV / GSLV S2</t>
+        </is>
+      </c>
+      <c r="C38" s="40" t="inlineStr">
+        <is>
+          <t>NTO/UDMH</t>
+        </is>
+      </c>
+      <c r="D38" s="40" t="n">
+        <v>293</v>
+      </c>
+      <c r="E38" s="40" t="n">
+        <v>270</v>
+      </c>
+      <c r="F38" s="40" t="n">
+        <v>800</v>
+      </c>
+      <c r="G38" s="40" t="n">
+        <v>725</v>
+      </c>
+      <c r="H38" s="40" t="n">
+        <v>634</v>
+      </c>
+      <c r="I38" s="40" t="n">
+        <v>58</v>
+      </c>
+      <c r="J38" s="40" t="n">
+        <v>16</v>
+      </c>
+      <c r="K38" s="39" t="inlineStr">
+        <is>
+          <t>Indian engine; Ariane Viking derivative</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="15" customHeight="1">
+      <c r="A39" s="39" t="inlineStr">
+        <is>
           <t>YF-20 (cluster)</t>
         </is>
       </c>
-      <c r="B38" s="39" t="inlineStr">
+      <c r="B39" s="39" t="inlineStr">
         <is>
           <t>Long March S1</t>
         </is>
       </c>
-      <c r="C38" s="40" t="inlineStr">
+      <c r="C39" s="40" t="inlineStr">
         <is>
           <t>NTO/UDMH</t>
         </is>
       </c>
-      <c r="D38" s="40" t="n">
+      <c r="D39" s="40" t="n">
         <v>289</v>
       </c>
-      <c r="E38" s="40" t="n">
+      <c r="E39" s="40" t="n">
         <v>259</v>
       </c>
-      <c r="F38" s="40" t="n">
+      <c r="F39" s="40" t="n">
         <v>2962</v>
       </c>
-      <c r="G38" s="40" t="n">
+      <c r="G39" s="40" t="n">
         <v>2799</v>
       </c>
-      <c r="H38" s="40" t="n">
+      <c r="H39" s="40" t="n">
         <v>4000</v>
       </c>
-      <c r="I38" s="40" t="n">
+      <c r="I39" s="40" t="n">
         <v>65</v>
       </c>
-      <c r="J38" s="40" t="n">
+      <c r="J39" s="40" t="n">
         <v>14</v>
       </c>
-      <c r="K38" s="39" t="inlineStr">
+      <c r="K39" s="39" t="inlineStr">
         <is>
           <t>4-chamber cluster used on CZ-2/3/4 first stages</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="7" t="inlineStr">
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>── Solid HTPB ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="15" customHeight="1">
-      <c r="A40" s="39" t="inlineStr">
-        <is>
-          <t>SRB (SLS 5-seg)</t>
-        </is>
-      </c>
-      <c r="B40" s="39" t="inlineStr">
-        <is>
-          <t>SLS Block 1</t>
-        </is>
-      </c>
-      <c r="C40" s="40" t="inlineStr">
-        <is>
-          <t>Solid HTPB</t>
-        </is>
-      </c>
-      <c r="D40" s="40" t="n">
-        <v>269</v>
-      </c>
-      <c r="E40" s="40" t="n">
-        <v>242</v>
-      </c>
-      <c r="F40" s="40" t="n">
-        <v>16000</v>
-      </c>
-      <c r="G40" s="40" t="n">
-        <v>14900</v>
-      </c>
-      <c r="H40" s="40" t="n">
-        <v>90718</v>
-      </c>
-      <c r="I40" s="40" t="n">
-        <v>62</v>
-      </c>
-      <c r="J40" s="40" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="K40" s="39" t="inlineStr">
-        <is>
-          <t>Largest SRB ever flown; 2x on SLS</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="39" t="inlineStr">
         <is>
-          <t>RSRM (Shuttle)</t>
+          <t>SRB (SLS 5-seg)</t>
         </is>
       </c>
       <c r="B41" s="39" t="inlineStr">
         <is>
-          <t>Space Shuttle</t>
+          <t>SLS Block 1</t>
         </is>
       </c>
       <c r="C41" s="40" t="inlineStr">
@@ -3939,41 +4050,41 @@
         </is>
       </c>
       <c r="D41" s="40" t="n">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E41" s="40" t="n">
         <v>242</v>
       </c>
       <c r="F41" s="40" t="n">
-        <v>14678</v>
+        <v>16000</v>
       </c>
       <c r="G41" s="40" t="n">
-        <v>12453</v>
+        <v>14900</v>
       </c>
       <c r="H41" s="40" t="n">
-        <v>90714</v>
+        <v>90718</v>
       </c>
       <c r="I41" s="40" t="n">
         <v>62</v>
       </c>
       <c r="J41" s="40" t="n">
-        <v>7.7</v>
+        <v>7.5</v>
       </c>
       <c r="K41" s="39" t="inlineStr">
         <is>
-          <t>4-segment Shuttle SRB</t>
+          <t>Largest SRB ever flown; 2x on SLS</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="39" t="inlineStr">
         <is>
-          <t>GEM-63XL</t>
+          <t>RSRM (Shuttle)</t>
         </is>
       </c>
       <c r="B42" s="39" t="inlineStr">
         <is>
-          <t>Vulcan strap-on</t>
+          <t>Space Shuttle</t>
         </is>
       </c>
       <c r="C42" s="40" t="inlineStr">
@@ -3982,41 +4093,41 @@
         </is>
       </c>
       <c r="D42" s="40" t="n">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="E42" s="40" t="n">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="F42" s="40" t="n">
-        <v>2140</v>
+        <v>14678</v>
       </c>
       <c r="G42" s="40" t="n">
-        <v>1930</v>
+        <v>12453</v>
       </c>
       <c r="H42" s="40" t="n">
-        <v>7000</v>
+        <v>90714</v>
       </c>
       <c r="I42" s="40" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J42" s="40" t="n">
-        <v>11</v>
+        <v>7.7</v>
       </c>
       <c r="K42" s="39" t="inlineStr">
         <is>
-          <t>Solid strap-on; also used on Atlas V 500</t>
+          <t>4-segment Shuttle SRB</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="39" t="inlineStr">
         <is>
-          <t>P80</t>
+          <t>GEM-63XL</t>
         </is>
       </c>
       <c r="B43" s="39" t="inlineStr">
         <is>
-          <t>Ariane 6 S1</t>
+          <t>Vulcan strap-on</t>
         </is>
       </c>
       <c r="C43" s="40" t="inlineStr">
@@ -4025,41 +4136,41 @@
         </is>
       </c>
       <c r="D43" s="40" t="n">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E43" s="40" t="n">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="F43" s="40" t="n">
-        <v>3040</v>
+        <v>2140</v>
       </c>
       <c r="G43" s="40" t="n">
-        <v>2820</v>
+        <v>1930</v>
       </c>
       <c r="H43" s="40" t="n">
-        <v>5650</v>
+        <v>7000</v>
       </c>
       <c r="I43" s="40" t="n">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="J43" s="40" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="K43" s="39" t="inlineStr">
         <is>
-          <t>Ariane 6 first stage solid motor</t>
+          <t>Solid strap-on; also used on Atlas V 500</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="39" t="inlineStr">
         <is>
-          <t>Zefiro-23</t>
+          <t>P80</t>
         </is>
       </c>
       <c r="B44" s="39" t="inlineStr">
         <is>
-          <t>Vega S2</t>
+          <t>Ariane 6 S1</t>
         </is>
       </c>
       <c r="C44" s="40" t="inlineStr">
@@ -4068,45 +4179,41 @@
         </is>
       </c>
       <c r="D44" s="40" t="n">
-        <v>287</v>
-      </c>
-      <c r="E44" s="40" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>278</v>
+      </c>
+      <c r="E44" s="40" t="n">
+        <v>255</v>
       </c>
       <c r="F44" s="40" t="n">
-        <v>1120</v>
-      </c>
-      <c r="G44" s="40" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>3040</v>
+      </c>
+      <c r="G44" s="40" t="n">
+        <v>2820</v>
       </c>
       <c r="H44" s="40" t="n">
-        <v>1315</v>
+        <v>5650</v>
       </c>
       <c r="I44" s="40" t="n">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="J44" s="40" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="K44" s="39" t="inlineStr">
         <is>
-          <t>Vega second stage solid motor</t>
+          <t>Ariane 6 first stage solid motor</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="39" t="inlineStr">
         <is>
-          <t>Zefiro-9</t>
+          <t>Zefiro-23</t>
         </is>
       </c>
       <c r="B45" s="39" t="inlineStr">
         <is>
-          <t>Vega S3</t>
+          <t>Vega S2</t>
         </is>
       </c>
       <c r="C45" s="40" t="inlineStr">
@@ -4115,7 +4222,7 @@
         </is>
       </c>
       <c r="D45" s="40" t="n">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="E45" s="40" t="inlineStr">
         <is>
@@ -4123,7 +4230,7 @@
         </is>
       </c>
       <c r="F45" s="40" t="n">
-        <v>314</v>
+        <v>1120</v>
       </c>
       <c r="G45" s="40" t="inlineStr">
         <is>
@@ -4131,29 +4238,29 @@
         </is>
       </c>
       <c r="H45" s="40" t="n">
-        <v>260</v>
+        <v>1315</v>
       </c>
       <c r="I45" s="40" t="n">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J45" s="40" t="n">
-        <v>54</v>
+        <v>30</v>
       </c>
       <c r="K45" s="39" t="inlineStr">
         <is>
-          <t>Vega third stage solid motor</t>
+          <t>Vega second stage solid motor</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="39" t="inlineStr">
         <is>
-          <t>Star-48BV</t>
+          <t>Zefiro-9</t>
         </is>
       </c>
       <c r="B46" s="39" t="inlineStr">
         <is>
-          <t>Various kick stages</t>
+          <t>Vega S3</t>
         </is>
       </c>
       <c r="C46" s="40" t="inlineStr">
@@ -4162,7 +4269,7 @@
         </is>
       </c>
       <c r="D46" s="40" t="n">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="E46" s="40" t="inlineStr">
         <is>
@@ -4170,7 +4277,7 @@
         </is>
       </c>
       <c r="F46" s="40" t="n">
-        <v>68</v>
+        <v>314</v>
       </c>
       <c r="G46" s="40" t="inlineStr">
         <is>
@@ -4178,62 +4285,109 @@
         </is>
       </c>
       <c r="H46" s="40" t="n">
-        <v>119</v>
+        <v>260</v>
       </c>
       <c r="I46" s="40" t="n">
-        <v>40</v>
+        <v>98</v>
       </c>
       <c r="J46" s="40" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K46" s="39" t="inlineStr">
         <is>
-          <t>Small solid kick motor; spin-stabilized</t>
+          <t>Vega third stage solid motor</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="39" t="inlineStr">
         <is>
+          <t>Star-48BV</t>
+        </is>
+      </c>
+      <c r="B47" s="39" t="inlineStr">
+        <is>
+          <t>Various kick stages</t>
+        </is>
+      </c>
+      <c r="C47" s="40" t="inlineStr">
+        <is>
+          <t>Solid HTPB</t>
+        </is>
+      </c>
+      <c r="D47" s="40" t="n">
+        <v>292</v>
+      </c>
+      <c r="E47" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F47" s="40" t="n">
+        <v>68</v>
+      </c>
+      <c r="G47" s="40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" s="40" t="n">
+        <v>119</v>
+      </c>
+      <c r="I47" s="40" t="n">
+        <v>40</v>
+      </c>
+      <c r="J47" s="40" t="n">
+        <v>55</v>
+      </c>
+      <c r="K47" s="39" t="inlineStr">
+        <is>
+          <t>Small solid kick motor; spin-stabilized</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="15" customHeight="1">
+      <c r="A48" s="39" t="inlineStr">
+        <is>
           <t>Castor 30B</t>
         </is>
       </c>
-      <c r="B47" s="39" t="inlineStr">
+      <c r="B48" s="39" t="inlineStr">
         <is>
           <t>Antares S2</t>
         </is>
       </c>
-      <c r="C47" s="40" t="inlineStr">
+      <c r="C48" s="40" t="inlineStr">
         <is>
           <t>Solid HTPB</t>
         </is>
       </c>
-      <c r="D47" s="40" t="n">
+      <c r="D48" s="40" t="n">
         <v>302</v>
       </c>
-      <c r="E47" s="40" t="inlineStr">
+      <c r="E48" s="40" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F47" s="40" t="n">
+      <c r="F48" s="40" t="n">
         <v>357</v>
       </c>
-      <c r="G47" s="40" t="inlineStr">
+      <c r="G48" s="40" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H47" s="40" t="n">
+      <c r="H48" s="40" t="n">
         <v>1437</v>
       </c>
-      <c r="I47" s="40" t="n">
+      <c r="I48" s="40" t="n">
         <v>80</v>
       </c>
-      <c r="J47" s="40" t="n">
+      <c r="J48" s="40" t="n">
         <v>57</v>
       </c>
-      <c r="K47" s="39" t="inlineStr">
+      <c r="K48" s="39" t="inlineStr">
         <is>
           <t>Antares second stage solid motor</t>
         </is>
@@ -4242,13 +4396,13 @@
   </sheetData>
   <autoFilter ref="A2:K2"/>
   <mergeCells count="7">
+    <mergeCell ref="A34:K34"/>
     <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A39:K39"/>
     <mergeCell ref="A15:K15"/>
-    <mergeCell ref="A33:K33"/>
     <mergeCell ref="A28:K28"/>
-    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="A40:K40"/>
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A37:K37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
improvements to gravity loss model
</commit_message>
<xml_diff>
--- a/launch_vehicle_design.xlsx
+++ b/launch_vehicle_design.xlsx
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M80"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -805,7 +805,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>New Glenn Block 2 (7x2)</t>
+          <t>Falcon 9 Block 5 (ASDS)</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>LEO 400km</t>
+          <t>LEO 400km / GTO</t>
         </is>
       </c>
     </row>
@@ -877,131 +877,119 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>← Gravity loss = coeff / TWR_liftoff; calibrated to ~1450 m/s at TWR=1.2; adjust to match known vehicles</t>
+          <t>← Base gravity loss = coeff / TWR_liftoff (trajectory-independent term); ~1750 typical</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>GTO Orbital ΔV</t>
+          <t>LEO Trajectory Penalty</t>
         </is>
       </c>
       <c r="B12" s="10" t="n">
-        <v>10400</v>
+        <v>500</v>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>← Velocity needed at GTO perigee — ~10,200-10,500 m/s depending on inclination and target apogee</t>
+          <t>← Extra gravity loss for LEO recovery pitch profile; 0=expendable, ~500=ASDS, ~900=RTLS</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
+          <t>GTO Trajectory Penalty</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>← Extra gravity loss for GTO pitch profile; smaller than LEO — S1 burns less time/downrange; ~0-150 m/s typical</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>GTO Orbital ΔV</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>10400</v>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>← Velocity needed at GTO perigee — ~10,200-10,500 m/s depending on inclination and target apogee</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
           <t>Number of Stages</t>
         </is>
       </c>
-      <c r="B13" s="9" t="n">
+      <c r="B15" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>← Active stages (enter 1-3)</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>STAGE CONFIGURATION</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>Stage Name</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>S1 First</t>
-        </is>
-      </c>
-      <c r="H16" s="9" t="inlineStr">
-        <is>
-          <t>S2 Upper</t>
-        </is>
-      </c>
-      <c r="K16" s="9" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Engine (from Engine DB)</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>BE-4 Block 2</t>
-        </is>
-      </c>
-      <c r="H17" s="9" t="inlineStr">
-        <is>
-          <t>BE-3U Block 2</t>
-        </is>
-      </c>
-      <c r="K17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Number of Engines</t>
+          <t>Stage Name</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="n">
-        <v>7</v>
-      </c>
-      <c r="H18" s="9" t="n">
-        <v>2</v>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>S1 Core</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>S2 Upper</t>
+        </is>
       </c>
       <c r="K18" s="9" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Propellant Combination</t>
+          <t>Engine (from Engine DB)</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>name</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>LOX/CH4</t>
+          <t>Merlin 1D</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>LOX/LH2</t>
+          <t>Merlin 1D Vac</t>
         </is>
       </c>
       <c r="K19" s="9" t="inlineStr"/>
@@ -1009,47 +997,49 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Propellant Mass (nominal)</t>
+          <t>Number of Engines</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="n">
-        <v>770000</v>
-      </c>
-      <c r="H20" s="10" t="n">
-        <v>75000</v>
-      </c>
-      <c r="K20" s="10" t="inlineStr"/>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Subcooling Gain (%)</t>
+          <t>Propellant Combination</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="H21" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="9" t="n">
-        <v>0</v>
-      </c>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>LOX/RP-1</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>LOX/RP-1</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Effective Propellant Mass</t>
+          <t>Propellant Mass (nominal)</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -1057,44 +1047,39 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E22" s="13">
-        <f>IFERROR(E20*(1+E21/100),"")</f>
-        <v/>
-      </c>
-      <c r="H22" s="13">
-        <f>IFERROR(H20*(1+H21/100),"")</f>
-        <v/>
-      </c>
-      <c r="K22" s="13">
-        <f>IFERROR(K20*(1+K21/100),"")</f>
-        <v/>
-      </c>
+      <c r="E22" s="10" t="n">
+        <v>411000</v>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>111500</v>
+      </c>
+      <c r="K22" s="10" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Recovery ΔV Reserve (m/s)</t>
+          <t>Subcooling Gain (%)</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>m/s</t>
-        </is>
-      </c>
-      <c r="E23" s="10" t="n">
-        <v>500</v>
-      </c>
-      <c r="H23" s="10" t="n">
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="10" t="n">
+      <c r="H23" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>Recovery Propellant Reserved</t>
+          <t>Effective Propellant Mass</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
@@ -1102,105 +1087,111 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E24" s="14">
-        <f>IFERROR(IF(E23=0,0,E58*(EXP(E23/(E28*9.80665))-1)),0)</f>
-        <v/>
-      </c>
-      <c r="H24" s="14">
-        <f>IFERROR(IF(H23=0,0,H58*(EXP(H23/(H28*9.80665))-1)),0)</f>
-        <v/>
-      </c>
-      <c r="K24" s="14">
-        <f>IFERROR(IF(K23=0,0,K58*(EXP(K23/(K28*9.80665))-1)),0)</f>
+      <c r="E24" s="13">
+        <f>IFERROR(E22*(1+E23/100),"")</f>
+        <v/>
+      </c>
+      <c r="H24" s="13">
+        <f>IFERROR(H22*(1+H23/100),"")</f>
+        <v/>
+      </c>
+      <c r="K24" s="13">
+        <f>IFERROR(K22*(1+K23/100),"")</f>
         <v/>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>LEO ΔV Fraction</t>
+          <t>Recovery ΔV Reserve (m/s)</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>0-1</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="n">
-        <v>0.597</v>
-      </c>
-      <c r="H25" s="9" t="n">
-        <v>0.403</v>
-      </c>
-      <c r="K25" s="9" t="inlineStr"/>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="H25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>LEO ΔV Allocation</t>
+          <t>Recovery Propellant Reserved</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>m/s</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E26" s="14">
-        <f>IFERROR(E25*B39,"")</f>
+        <f>IFERROR(IF(E25=0,0,E61*(EXP(E25/(E30*9.80665))-1)),0)</f>
         <v/>
       </c>
       <c r="H26" s="14">
-        <f>IFERROR(H25*B39,"")</f>
+        <f>IFERROR(IF(H25=0,0,H61*(EXP(H25/(H30*9.80665))-1)),0)</f>
         <v/>
       </c>
       <c r="K26" s="14">
-        <f>IFERROR(K25*B39,"")</f>
+        <f>IFERROR(IF(K25=0,0,K61*(EXP(K25/(K30*9.80665))-1)),0)</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Vac Isp Override</t>
+          <t>LEO ΔV Fraction</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="inlineStr"/>
-      <c r="H27" s="9" t="inlineStr"/>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>0.6</v>
+      </c>
       <c r="K27" s="9" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>Vac Isp (from DB)</t>
+          <t>LEO ΔV Allocation</t>
         </is>
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="E28" s="15">
-        <f>IF(E27&lt;&gt;"",E27,IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
-        <v/>
-      </c>
-      <c r="H28" s="15">
-        <f>IF(H27&lt;&gt;"",H27,IFERROR(VLOOKUP(H17,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
-        <v/>
-      </c>
-      <c r="K28" s="15">
-        <f>IF(K27&lt;&gt;"",K27,IFERROR(VLOOKUP(K17,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="E28" s="14">
+        <f>IFERROR(E27*B42,"")</f>
+        <v/>
+      </c>
+      <c r="H28" s="14">
+        <f>IFERROR(H27*B42,"")</f>
+        <v/>
+      </c>
+      <c r="K28" s="14">
+        <f>IFERROR(K27*B42,"")</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>SL Isp (from DB)</t>
+          <t>Vac Isp Override</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
@@ -1208,44 +1199,38 @@
           <t>s</t>
         </is>
       </c>
-      <c r="E29" s="15">
-        <f>IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,5,0),"—")</f>
-        <v/>
-      </c>
-      <c r="H29" s="15">
-        <f>IFERROR(VLOOKUP(H17,'Engine DB'!$A:$K,5,0),"—")</f>
-        <v/>
-      </c>
-      <c r="K29" s="15">
-        <f>IFERROR(VLOOKUP(K17,'Engine DB'!$A:$K,5,0),"—")</f>
-        <v/>
-      </c>
+      <c r="E29" s="9" t="inlineStr"/>
+      <c r="H29" s="9" t="inlineStr"/>
+      <c r="K29" s="9" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Atm Fraction (0-1)</t>
+          <t>Vac Isp (from DB)</t>
         </is>
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E30" s="9" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H30" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="K30" s="9" t="n">
-        <v>1</v>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E30" s="15">
+        <f>IF(E29&lt;&gt;"",E29,IFERROR(VLOOKUP(E19,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+        <v/>
+      </c>
+      <c r="H30" s="15">
+        <f>IF(H29&lt;&gt;"",H29,IFERROR(VLOOKUP(H19,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+        <v/>
+      </c>
+      <c r="K30" s="15">
+        <f>IF(K29&lt;&gt;"",K29,IFERROR(VLOOKUP(K19,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+        <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Effective Isp (used)</t>
+          <t>SL Isp (from DB)</t>
         </is>
       </c>
       <c r="B31" s="12" t="inlineStr">
@@ -1253,246 +1238,230 @@
           <t>s</t>
         </is>
       </c>
-      <c r="E31" s="16">
-        <f>IFERROR(IF(ISNUMBER(E29),E29+E30*(E28-E29),E28),E28)</f>
-        <v/>
-      </c>
-      <c r="H31" s="16">
-        <f>IFERROR(IF(ISNUMBER(H29),H29+H30*(H28-H29),H28),H28)</f>
-        <v/>
-      </c>
-      <c r="K31" s="16">
-        <f>IFERROR(IF(ISNUMBER(K29),K29+K30*(K28-K29),K28),K28)</f>
+      <c r="E31" s="15">
+        <f>IFERROR(VLOOKUP(E19,'Engine DB'!$A:$K,5,0),"—")</f>
+        <v/>
+      </c>
+      <c r="H31" s="15">
+        <f>IFERROR(VLOOKUP(H19,'Engine DB'!$A:$K,5,0),"—")</f>
+        <v/>
+      </c>
+      <c r="K31" s="15">
+        <f>IFERROR(VLOOKUP(K19,'Engine DB'!$A:$K,5,0),"—")</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>GTO ΔV Fraction</t>
+          <t>Atm Fraction (0-1)</t>
         </is>
       </c>
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E32" s="9" t="n">
-        <v>0.555</v>
+        <v>0.6</v>
       </c>
       <c r="H32" s="9" t="n">
-        <v>0.445</v>
-      </c>
-      <c r="K32" s="9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="K32" s="9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
+          <t>Effective Isp (used)</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E33" s="16">
+        <f>IFERROR(IF(ISNUMBER(E31),E31+E32*(E30-E31),E30),E30)</f>
+        <v/>
+      </c>
+      <c r="H33" s="16">
+        <f>IFERROR(IF(ISNUMBER(H31),H31+H32*(H30-H31),H30),H30)</f>
+        <v/>
+      </c>
+      <c r="K33" s="16">
+        <f>IFERROR(IF(ISNUMBER(K31),K31+K32*(K30-K31),K30),K30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>GTO ΔV Fraction</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="H34" s="9" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="K34" s="9" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
           <t>GTO ΔV Allocation</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>m/s</t>
         </is>
       </c>
-      <c r="E33" s="14">
-        <f>IFERROR(E32*B40,"")</f>
-        <v/>
-      </c>
-      <c r="H33" s="14">
-        <f>IFERROR(H32*B40,"")</f>
-        <v/>
-      </c>
-      <c r="K33" s="14">
-        <f>IFERROR(K32*B40,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="7" t="inlineStr">
+      <c r="E35" s="14">
+        <f>IFERROR(E34*B43,"")</f>
+        <v/>
+      </c>
+      <c r="H35" s="14">
+        <f>IFERROR(H34*B43,"")</f>
+        <v/>
+      </c>
+      <c r="K35" s="14">
+        <f>IFERROR(K34*B43,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>MISSION ΔV ANALYSIS  —  Gravity loss computed from liftoff TWR</t>
         </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>Est. GLOW (stage masses only, no payload)</t>
-        </is>
-      </c>
-      <c r="B36" s="14">
-        <f>IFERROR(E20+E58,0)+IFERROR(H20+H58,0)+IFERROR(K20+K58,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>Stage 1 Liftoff TWR (est., no payload)</t>
-        </is>
-      </c>
-      <c r="B37" s="17">
-        <f>IFERROR(E18*IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,7,0),0)*1000/(B36*9.80665),"")</f>
-        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>Gravity Loss (= coeff / TWR)</t>
+          <t>Est. GLOW (stage masses only, no payload)</t>
         </is>
       </c>
       <c r="B38" s="14">
-        <f>IFERROR(B11/B37,"")</f>
+        <f>IFERROR(E22+E61,0)+IFERROR(H22+H61,0)+IFERROR(K22+K61,0)</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>LEO Mission ΔV (calculated)</t>
-        </is>
-      </c>
-      <c r="B39" s="18">
-        <f>IFERROR(B9+B10+B38,"")</f>
+          <t>Stage 1 Liftoff TWR (est., no payload)</t>
+        </is>
+      </c>
+      <c r="B39" s="17">
+        <f>IFERROR(E20*IFERROR(VLOOKUP(E19,'Engine DB'!$A:$K,7,0),0)*1000/(B38*9.80665),"")</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>GTO Mission ΔV (calculated)</t>
-        </is>
-      </c>
-      <c r="B40" s="18">
-        <f>IFERROR(B12+B10+B38,"")</f>
+          <t>LEO Gravity Loss (= coeff / TWR + LEO penalty)</t>
+        </is>
+      </c>
+      <c r="B40" s="14">
+        <f>IFERROR(B11/B39+B12,"")</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="19" t="inlineStr">
-        <is>
-          <t>LEO ΔV Allocation Check (should = LEO Mission ΔV above)</t>
-        </is>
-      </c>
-      <c r="B41" s="20">
-        <f>IFERROR(E26*1,0)+IFERROR(H26*1,0)+IFERROR(K26*1,0)</f>
-        <v/>
-      </c>
-      <c r="C41" s="2">
-        <f>IF(ABS(B41-B39)&lt;1,"✓ OK","⚠ Adjust stage allocations to sum to LEO Mission ΔV")</f>
+      <c r="A41" s="8" t="inlineStr">
+        <is>
+          <t>GTO Gravity Loss (= coeff / TWR + GTO penalty)</t>
+        </is>
+      </c>
+      <c r="B41" s="14">
+        <f>IFERROR(B11/B39+B13,"")</f>
         <v/>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
         <is>
+          <t>LEO Mission ΔV (calculated)</t>
+        </is>
+      </c>
+      <c r="B42" s="18">
+        <f>IFERROR(B9+B10+B40,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="inlineStr">
+        <is>
+          <t>GTO Mission ΔV (calculated)</t>
+        </is>
+      </c>
+      <c r="B43" s="18">
+        <f>IFERROR(B14+B10+B41,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="19" t="inlineStr">
+        <is>
+          <t>LEO ΔV Allocation Check (should = LEO Mission ΔV above)</t>
+        </is>
+      </c>
+      <c r="B44" s="20">
+        <f>IFERROR(E28*1,0)+IFERROR(H28*1,0)+IFERROR(K28*1,0)</f>
+        <v/>
+      </c>
+      <c r="C44" s="2">
+        <f>IF(ABS(B44-B42)&lt;1,"✓ OK","⚠ Adjust stage allocations to sum to LEO Mission ΔV")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="inlineStr">
+        <is>
           <t>Engine Mass per Engine</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
+      <c r="B45" s="12" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E42" s="21">
-        <f>IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,8,0),"—")</f>
-        <v/>
-      </c>
-      <c r="H42" s="21">
-        <f>IFERROR(VLOOKUP(H17,'Engine DB'!$A:$K,8,0),"—")</f>
-        <v/>
-      </c>
-      <c r="K42" s="21">
-        <f>IFERROR(VLOOKUP(K17,'Engine DB'!$A:$K,8,0),"—")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="7" t="inlineStr">
+      <c r="E45" s="21">
+        <f>IFERROR(VLOOKUP(E19,'Engine DB'!$A:$K,8,0),"—")</f>
+        <v/>
+      </c>
+      <c r="H45" s="21">
+        <f>IFERROR(VLOOKUP(H19,'Engine DB'!$A:$K,8,0),"—")</f>
+        <v/>
+      </c>
+      <c r="K45" s="21">
+        <f>IFERROR(VLOOKUP(K19,'Engine DB'!$A:$K,8,0),"—")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="7" t="inlineStr">
         <is>
           <t>SUBSYSTEM MASS BREAKDOWN (auto-estimated; override any yellow cell)</t>
         </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="22" t="inlineStr">
-        <is>
-          <t>Tank Structure</t>
-        </is>
-      </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E45" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",3.5,IF(E19="LOX/LH2",6.5,IF(E19="LOX/CH4",3.8,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),1.8,2.5)))))</f>
-        <v/>
-      </c>
-      <c r="H45" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",3.5,IF(H19="LOX/LH2",6.5,IF(H19="LOX/CH4",3.8,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),1.8,2.5)))))</f>
-        <v/>
-      </c>
-      <c r="K45" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",3.5,IF(K19="LOX/LH2",6.5,IF(K19="LOX/CH4",3.8,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),1.8,2.5)))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="22" t="inlineStr">
-        <is>
-          <t>Pressurization System</t>
-        </is>
-      </c>
-      <c r="B46" s="12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E46" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.4,IF(E19="LOX/LH2",0.6,IF(E19="LOX/CH4",0.4,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="H46" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.4,IF(H19="LOX/LH2",0.6,IF(H19="LOX/CH4",0.4,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.0,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="K46" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.4,IF(K19="LOX/LH2",0.6,IF(K19="LOX/CH4",0.4,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.0,0.5)))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="22" t="inlineStr">
-        <is>
-          <t>Feed System / Plumbing</t>
-        </is>
-      </c>
-      <c r="B47" s="12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E47" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.8,IF(E19="LOX/LH2",1.0,IF(E19="LOX/CH4",0.8,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.2,0.6)))))</f>
-        <v/>
-      </c>
-      <c r="H47" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.8,IF(H19="LOX/LH2",1.0,IF(H19="LOX/CH4",0.8,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.2,0.6)))))</f>
-        <v/>
-      </c>
-      <c r="K47" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.8,IF(K19="LOX/LH2",1.0,IF(K19="LOX/CH4",0.8,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.2,0.6)))))</f>
-        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="22" t="inlineStr">
         <is>
-          <t>Avionics / GNC</t>
+          <t>Tank Structure</t>
         </is>
       </c>
       <c r="B48" s="12" t="inlineStr">
@@ -1501,22 +1470,22 @@
         </is>
       </c>
       <c r="E48" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.3,IF(E19="LOX/LH2",0.4,IF(E19="LOX/CH4",0.3,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.2,0.4)))))</f>
+        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",3.5,IF(E21="LOX/LH2",6.5,IF(E21="LOX/CH4",3.8,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),1.8,2.5)))))</f>
         <v/>
       </c>
       <c r="H48" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.3,IF(H19="LOX/LH2",0.4,IF(H19="LOX/CH4",0.3,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.2,0.4)))))</f>
+        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",3.5,IF(H21="LOX/LH2",6.5,IF(H21="LOX/CH4",3.8,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),1.8,2.5)))))</f>
         <v/>
       </c>
       <c r="K48" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.3,IF(K19="LOX/LH2",0.4,IF(K19="LOX/CH4",0.3,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.2,0.4)))))</f>
+        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",3.5,IF(K21="LOX/LH2",6.5,IF(K21="LOX/CH4",3.8,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),1.8,2.5)))))</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="22" t="inlineStr">
         <is>
-          <t>Power System</t>
+          <t>Pressurization System</t>
         </is>
       </c>
       <c r="B49" s="12" t="inlineStr">
@@ -1525,22 +1494,22 @@
         </is>
       </c>
       <c r="E49" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.2,IF(E19="LOX/LH2",0.3,IF(E19="LOX/CH4",0.2,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.4,IF(E21="LOX/LH2",0.6,IF(E21="LOX/CH4",0.4,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.0,0.5)))))</f>
         <v/>
       </c>
       <c r="H49" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.2,IF(H19="LOX/LH2",0.3,IF(H19="LOX/CH4",0.2,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.4,IF(H21="LOX/LH2",0.6,IF(H21="LOX/CH4",0.4,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.0,0.5)))))</f>
         <v/>
       </c>
       <c r="K49" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.2,IF(K19="LOX/LH2",0.3,IF(K19="LOX/CH4",0.2,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.4,IF(K21="LOX/LH2",0.6,IF(K21="LOX/CH4",0.4,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.0,0.5)))))</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="22" t="inlineStr">
         <is>
-          <t>Thermal Control</t>
+          <t>Feed System / Plumbing</t>
         </is>
       </c>
       <c r="B50" s="12" t="inlineStr">
@@ -1549,22 +1518,22 @@
         </is>
       </c>
       <c r="E50" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.2,IF(E19="LOX/LH2",1.0,IF(E19="LOX/CH4",0.3,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.1,0.3)))))</f>
+        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.8,IF(E21="LOX/LH2",1.0,IF(E21="LOX/CH4",0.8,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.2,0.6)))))</f>
         <v/>
       </c>
       <c r="H50" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.2,IF(H19="LOX/LH2",1.0,IF(H19="LOX/CH4",0.3,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.1,0.3)))))</f>
+        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.8,IF(H21="LOX/LH2",1.0,IF(H21="LOX/CH4",0.8,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.2,0.6)))))</f>
         <v/>
       </c>
       <c r="K50" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.2,IF(K19="LOX/LH2",1.0,IF(K19="LOX/CH4",0.3,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.1,0.3)))))</f>
+        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.8,IF(K21="LOX/LH2",1.0,IF(K21="LOX/CH4",0.8,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.2,0.6)))))</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="22" t="inlineStr">
         <is>
-          <t>RCS / ACS</t>
+          <t>Avionics / GNC</t>
         </is>
       </c>
       <c r="B51" s="12" t="inlineStr">
@@ -1573,22 +1542,22 @@
         </is>
       </c>
       <c r="E51" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.3,IF(E19="LOX/LH2",0.4,IF(E19="LOX/CH4",0.3,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.3,IF(E21="LOX/LH2",0.4,IF(E21="LOX/CH4",0.3,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.2,0.4)))))</f>
         <v/>
       </c>
       <c r="H51" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.3,IF(H19="LOX/LH2",0.4,IF(H19="LOX/CH4",0.3,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.3,IF(H21="LOX/LH2",0.4,IF(H21="LOX/CH4",0.3,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.2,0.4)))))</f>
         <v/>
       </c>
       <c r="K51" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.3,IF(K19="LOX/LH2",0.4,IF(K19="LOX/CH4",0.3,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.3,IF(K21="LOX/LH2",0.4,IF(K21="LOX/CH4",0.3,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.2,0.4)))))</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="22" t="inlineStr">
         <is>
-          <t>Separation System</t>
+          <t>Power System</t>
         </is>
       </c>
       <c r="B52" s="12" t="inlineStr">
@@ -1597,22 +1566,22 @@
         </is>
       </c>
       <c r="E52" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.1,IF(E19="LOX/LH2",0.1,IF(E19="LOX/CH4",0.1,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.1,0.1)))))</f>
+        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.2,IF(E21="LOX/LH2",0.3,IF(E21="LOX/CH4",0.2,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
       <c r="H52" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.1,IF(H19="LOX/LH2",0.1,IF(H19="LOX/CH4",0.1,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.1,0.1)))))</f>
+        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.2,IF(H21="LOX/LH2",0.3,IF(H21="LOX/CH4",0.2,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
       <c r="K52" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.1,IF(K19="LOX/LH2",0.1,IF(K19="LOX/CH4",0.1,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.1,0.1)))))</f>
+        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.2,IF(K21="LOX/LH2",0.3,IF(K21="LOX/CH4",0.2,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="22" t="inlineStr">
         <is>
-          <t>Recovery Hardware</t>
+          <t>Thermal Control</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
@@ -1621,22 +1590,22 @@
         </is>
       </c>
       <c r="E53" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.0,IF(E19="LOX/LH2",0.0,IF(E19="LOX/CH4",0.0,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.0,0.0)))))</f>
+        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.2,IF(E21="LOX/LH2",1.0,IF(E21="LOX/CH4",0.3,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.1,0.3)))))</f>
         <v/>
       </c>
       <c r="H53" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.0,IF(H19="LOX/LH2",0.0,IF(H19="LOX/CH4",0.0,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.0,0.0)))))</f>
+        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.2,IF(H21="LOX/LH2",1.0,IF(H21="LOX/CH4",0.3,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.1,0.3)))))</f>
         <v/>
       </c>
       <c r="K53" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.0,IF(K19="LOX/LH2",0.0,IF(K19="LOX/CH4",0.0,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.0,0.0)))))</f>
+        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.2,IF(K21="LOX/LH2",1.0,IF(K21="LOX/CH4",0.3,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.1,0.3)))))</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="22" t="inlineStr">
         <is>
-          <t>Residuals / Margin</t>
+          <t>RCS / ACS</t>
         </is>
       </c>
       <c r="B54" s="12" t="inlineStr">
@@ -1645,459 +1614,537 @@
         </is>
       </c>
       <c r="E54" s="10">
-        <f>IF(E20="","",E20/100*IF(E19="LOX/RP-1",0.5,IF(E19="LOX/LH2",0.8,IF(E19="LOX/CH4",0.5,IF(OR(E19="Solid HTPB",E19="Solid PBAN"),0.3,0.5)))))</f>
+        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.3,IF(E21="LOX/LH2",0.4,IF(E21="LOX/CH4",0.3,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
       <c r="H54" s="10">
-        <f>IF(H20="","",H20/100*IF(H19="LOX/RP-1",0.5,IF(H19="LOX/LH2",0.8,IF(H19="LOX/CH4",0.5,IF(OR(H19="Solid HTPB",H19="Solid PBAN"),0.3,0.5)))))</f>
+        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.3,IF(H21="LOX/LH2",0.4,IF(H21="LOX/CH4",0.3,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
       <c r="K54" s="10">
-        <f>IF(K20="","",K20/100*IF(K19="LOX/RP-1",0.5,IF(K19="LOX/LH2",0.8,IF(K19="LOX/CH4",0.5,IF(OR(K19="Solid HTPB",K19="Solid PBAN"),0.3,0.5)))))</f>
+        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.3,IF(K21="LOX/LH2",0.4,IF(K21="LOX/CH4",0.3,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="22" t="inlineStr">
         <is>
+          <t>Separation System</t>
+        </is>
+      </c>
+      <c r="B55" s="12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E55" s="10">
+        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.1,IF(E21="LOX/LH2",0.1,IF(E21="LOX/CH4",0.1,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.1,0.1)))))</f>
+        <v/>
+      </c>
+      <c r="H55" s="10">
+        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.1,IF(H21="LOX/LH2",0.1,IF(H21="LOX/CH4",0.1,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.1,0.1)))))</f>
+        <v/>
+      </c>
+      <c r="K55" s="10">
+        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.1,IF(K21="LOX/LH2",0.1,IF(K21="LOX/CH4",0.1,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.1,0.1)))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="22" t="inlineStr">
+        <is>
+          <t>Recovery Hardware</t>
+        </is>
+      </c>
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E56" s="10">
+        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.0,IF(E21="LOX/LH2",0.0,IF(E21="LOX/CH4",0.0,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.0,0.0)))))</f>
+        <v/>
+      </c>
+      <c r="H56" s="10">
+        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.0,IF(H21="LOX/LH2",0.0,IF(H21="LOX/CH4",0.0,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.0,0.0)))))</f>
+        <v/>
+      </c>
+      <c r="K56" s="10">
+        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.0,IF(K21="LOX/LH2",0.0,IF(K21="LOX/CH4",0.0,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.0,0.0)))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="22" t="inlineStr">
+        <is>
+          <t>Residuals / Margin</t>
+        </is>
+      </c>
+      <c r="B57" s="12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E57" s="10">
+        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.5,IF(E21="LOX/LH2",0.8,IF(E21="LOX/CH4",0.5,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.3,0.5)))))</f>
+        <v/>
+      </c>
+      <c r="H57" s="10">
+        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.5,IF(H21="LOX/LH2",0.8,IF(H21="LOX/CH4",0.5,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.3,0.5)))))</f>
+        <v/>
+      </c>
+      <c r="K57" s="10">
+        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.5,IF(K21="LOX/LH2",0.8,IF(K21="LOX/CH4",0.5,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.3,0.5)))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="22" t="inlineStr">
+        <is>
           <t>Engine System Total</t>
         </is>
       </c>
-      <c r="B55" s="12" t="inlineStr">
+      <c r="B58" s="12" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E55" s="21">
-        <f>IFERROR(E18*E42*1.15, "")</f>
-        <v/>
-      </c>
-      <c r="H55" s="21">
-        <f>IFERROR(H18*H42*1.15, "")</f>
-        <v/>
-      </c>
-      <c r="K55" s="21">
-        <f>IFERROR(K18*K42*1.15, "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="23" t="inlineStr">
+      <c r="E58" s="21">
+        <f>IFERROR(E20*E45*1.15, "")</f>
+        <v/>
+      </c>
+      <c r="H58" s="21">
+        <f>IFERROR(H20*H45*1.15, "")</f>
+        <v/>
+      </c>
+      <c r="K58" s="21">
+        <f>IFERROR(K20*K45*1.15, "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="23" t="inlineStr">
         <is>
           <t>TOTAL DRY MASS (Estimated)</t>
         </is>
       </c>
-      <c r="B56" s="24" t="inlineStr">
+      <c r="B59" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E56" s="13">
-        <f>IFERROR(E45+E46+E47+E48+E49+E50+E51+E52+E53+E54+E55, "")</f>
-        <v/>
-      </c>
-      <c r="H56" s="13">
-        <f>IFERROR(H45+H46+H47+H48+H49+H50+H51+H52+H53+H54+H55, "")</f>
-        <v/>
-      </c>
-      <c r="K56" s="13">
-        <f>IFERROR(K45+K46+K47+K48+K49+K50+K51+K52+K53+K54+K55, "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="8" t="inlineStr">
+      <c r="E59" s="13">
+        <f>IFERROR(E48+E49+E50+E51+E52+E53+E54+E55+E56+E57+E58, "")</f>
+        <v/>
+      </c>
+      <c r="H59" s="13">
+        <f>IFERROR(H48+H49+H50+H51+H52+H53+H54+H55+H56+H57+H58, "")</f>
+        <v/>
+      </c>
+      <c r="K59" s="13">
+        <f>IFERROR(K48+K49+K50+K51+K52+K53+K54+K55+K56+K57+K58, "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
         <is>
           <t>Dry Mass Override (enter known value)</t>
         </is>
       </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="B60" s="12" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E57" s="10" t="inlineStr"/>
-      <c r="H57" s="10" t="inlineStr"/>
-      <c r="K57" s="10" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="E60" s="10" t="n">
+        <v>22200</v>
+      </c>
+      <c r="H60" s="10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K60" s="10" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
         <is>
           <t>Effective Dry Mass</t>
         </is>
       </c>
-      <c r="B58" s="12" t="inlineStr">
+      <c r="B61" s="12" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E58" s="21">
-        <f>IF(E57&lt;&gt;"",E57,E56)</f>
-        <v/>
-      </c>
-      <c r="H58" s="21">
-        <f>IF(H57&lt;&gt;"",H57,H56)</f>
-        <v/>
-      </c>
-      <c r="K58" s="21">
-        <f>IF(K57&lt;&gt;"",K57,K56)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="7" t="inlineStr">
-        <is>
-          <t>PERFORMANCE CALCULATIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="25" t="inlineStr">
-        <is>
-          <t>MAX PAYLOAD TO ORBIT</t>
-        </is>
-      </c>
-      <c r="B61" s="26">
-        <f>IF(B13&gt;=3,IFERROR((K22-K24)/(EXP(K26/(K31*9.80665))-1)-(K58+K24)-B8, ""),IF(B13&gt;=2,IFERROR((H22-H24)/(EXP(H26/(H31*9.80665))-1)-(H58+H24)-B8, ""),IFERROR((E22-E24)/(EXP(E26/(E31*9.80665))-1)-(E58+E24)-B8, "")))</f>
-        <v/>
-      </c>
-      <c r="C61" s="27" t="inlineStr">
-        <is>
-          <t>← Solved from last stage: m_payload = (prop−rec)/(e^(ΔV/Isp·g₀)−1) − (dry+rec) − adapter  |  Recovery penalty: lower stage's actual ΔV drops (see verification); reduce that stage's ΔV fraction to propagate penalty to payload</t>
-        </is>
+      <c r="E61" s="21">
+        <f>IF(E60&lt;&gt;"",E60,E59)</f>
+        <v/>
+      </c>
+      <c r="H61" s="21">
+        <f>IF(H60&lt;&gt;"",H60,H59)</f>
+        <v/>
+      </c>
+      <c r="K61" s="21">
+        <f>IF(K60&lt;&gt;"",K60,K59)</f>
+        <v/>
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>GTO PERFORMANCE</t>
+          <t>PERFORMANCE CALCULATIONS</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="25" t="inlineStr">
         <is>
+          <t>MAX PAYLOAD TO ORBIT</t>
+        </is>
+      </c>
+      <c r="B64" s="26">
+        <f>IF(B15&gt;=3,IFERROR((K24-K26)/(EXP(K28/(K33*9.80665))-1)-(K61+K26)-B8, ""),IF(B15&gt;=2,IFERROR((H24-H26)/(EXP(H28/(H33*9.80665))-1)-(H61+H26)-B8, ""),IFERROR((E24-E26)/(EXP(E28/(E33*9.80665))-1)-(E61+E26)-B8, "")))</f>
+        <v/>
+      </c>
+      <c r="C64" s="27" t="inlineStr">
+        <is>
+          <t>← Solved from last stage: m_payload = (prop−rec)/(e^(ΔV/Isp·g₀)−1) − (dry+rec) − adapter  |  Recovery penalty: lower stage's actual ΔV drops (see verification); reduce that stage's ΔV fraction to propagate penalty to payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>GTO PERFORMANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="25" t="inlineStr">
+        <is>
           <t>MAX PAYLOAD TO GTO</t>
         </is>
       </c>
-      <c r="B64" s="26">
-        <f>IF(B13&gt;=3,IFERROR((K22-K24)/(EXP(K33/(K31*9.80665))-1)-(K58+K24)-B8, ""),IF(B13&gt;=2,IFERROR((H22-H24)/(EXP(H33/(H31*9.80665))-1)-(H58+H24)-B8, ""),IFERROR((E22-E24)/(EXP(E33/(E31*9.80665))-1)-(E58+E24)-B8, "")))</f>
-        <v/>
-      </c>
-      <c r="C64" s="27" t="inlineStr">
+      <c r="B67" s="26">
+        <f>IF(B15&gt;=3,IFERROR((K24-K26)/(EXP(K35/(K33*9.80665))-1)-(K61+K26)-B8, ""),IF(B15&gt;=2,IFERROR((H24-H26)/(EXP(H35/(H33*9.80665))-1)-(H61+H26)-B8, ""),IFERROR((E24-E26)/(EXP(E35/(E33*9.80665))-1)-(E61+E26)-B8, "")))</f>
+        <v/>
+      </c>
+      <c r="C67" s="27" t="inlineStr">
         <is>
           <t>← MIN across all stage constraints using GTO ΔV allocations: capacity_i = (prop−rec)/(e^(ΔV/Isp·g₀)−1) − (dry+rec) − gross_above − adapter</t>
         </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="8" t="inlineStr">
-        <is>
-          <t>Gross Stage Mass (Prop + Dry)</t>
-        </is>
-      </c>
-      <c r="B65" s="12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E65" s="21">
-        <f>IFERROR(E22+E58, "")</f>
-        <v/>
-      </c>
-      <c r="H65" s="21">
-        <f>IFERROR(H22+H58, "")</f>
-        <v/>
-      </c>
-      <c r="K65" s="21">
-        <f>IFERROR(K22+K58, "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="8" t="inlineStr">
-        <is>
-          <t>Burnout Mass m_f</t>
-        </is>
-      </c>
-      <c r="B66" s="12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E66" s="21">
-        <f>IFERROR(E58+E24+IFERROR(H65*1,0)+IFERROR(K65*1,0)+B61+B8, "")</f>
-        <v/>
-      </c>
-      <c r="H66" s="21">
-        <f>IFERROR(H58+H24+IFERROR(K65*1,0)+B61+B8, "")</f>
-        <v/>
-      </c>
-      <c r="K66" s="21">
-        <f>IFERROR(K58+K24+B61+B8, "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="8" t="inlineStr">
-        <is>
-          <t>Initial Mass m_0 (at ignition)</t>
-        </is>
-      </c>
-      <c r="B67" s="12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E67" s="21">
-        <f>IFERROR(E66+E22-E24, "")</f>
-        <v/>
-      </c>
-      <c r="H67" s="21">
-        <f>IFERROR(H66+H22-H24, "")</f>
-        <v/>
-      </c>
-      <c r="K67" s="21">
-        <f>IFERROR(K66+K22-K24, "")</f>
-        <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>Mass Ratio (m₀ / m_f)</t>
+          <t>Gross Stage Mass (Prop + Dry)</t>
         </is>
       </c>
       <c r="B68" s="12" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E68" s="28">
-        <f>IFERROR(E67/E66, "")</f>
-        <v/>
-      </c>
-      <c r="H68" s="28">
-        <f>IFERROR(H67/H66, "")</f>
-        <v/>
-      </c>
-      <c r="K68" s="28">
-        <f>IFERROR(K67/K66, "")</f>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E68" s="21">
+        <f>IFERROR(E24+E61, "")</f>
+        <v/>
+      </c>
+      <c r="H68" s="21">
+        <f>IFERROR(H24+H61, "")</f>
+        <v/>
+      </c>
+      <c r="K68" s="21">
+        <f>IFERROR(K24+K61, "")</f>
         <v/>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="23" t="inlineStr">
-        <is>
-          <t>Actual Stage ΔV (verification)</t>
-        </is>
-      </c>
-      <c r="B69" s="24" t="inlineStr">
-        <is>
-          <t>m/s</t>
-        </is>
-      </c>
-      <c r="E69" s="13">
-        <f>IFERROR(E31*9.80665*LN(E68), "")</f>
-        <v/>
-      </c>
-      <c r="H69" s="13">
-        <f>IFERROR(H31*9.80665*LN(H68), "")</f>
-        <v/>
-      </c>
-      <c r="K69" s="13">
-        <f>IFERROR(K31*9.80665*LN(K68), "")</f>
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>Burnout Mass m_f</t>
+        </is>
+      </c>
+      <c r="B69" s="12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E69" s="21">
+        <f>IFERROR(E61+E26+IFERROR(H68*1,0)+IFERROR(K68*1,0)+B64+B8, "")</f>
+        <v/>
+      </c>
+      <c r="H69" s="21">
+        <f>IFERROR(H61+H26+IFERROR(K68*1,0)+B64+B8, "")</f>
+        <v/>
+      </c>
+      <c r="K69" s="21">
+        <f>IFERROR(K61+K26+B64+B8, "")</f>
         <v/>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
         <is>
-          <t>Thrust-to-Weight Ratio (at ignition)</t>
+          <t>Initial Mass m_0 (at ignition)</t>
         </is>
       </c>
       <c r="B70" s="12" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E70" s="29">
-        <f>IFERROR(E18*IFERROR(VLOOKUP(E17,'Engine DB'!$A:$K,7,0),0)*1000/(E67*9.80665), "")</f>
-        <v/>
-      </c>
-      <c r="H70" s="29">
-        <f>IFERROR(H18*IFERROR(VLOOKUP(H17,'Engine DB'!$A:$K,6,0),0)*1000/(H67*9.80665), "")</f>
-        <v/>
-      </c>
-      <c r="K70" s="29">
-        <f>IFERROR(K18*IFERROR(VLOOKUP(K17,'Engine DB'!$A:$K,6,0),0)*1000/(K67*9.80665), "")</f>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E70" s="21">
+        <f>IFERROR(E69+E24-E26, "")</f>
+        <v/>
+      </c>
+      <c r="H70" s="21">
+        <f>IFERROR(H69+H24-H26, "")</f>
+        <v/>
+      </c>
+      <c r="K70" s="21">
+        <f>IFERROR(K69+K24-K26, "")</f>
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
+          <t>Mass Ratio (m₀ / m_f)</t>
+        </is>
+      </c>
+      <c r="B71" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E71" s="28">
+        <f>IFERROR(E70/E69, "")</f>
+        <v/>
+      </c>
+      <c r="H71" s="28">
+        <f>IFERROR(H70/H69, "")</f>
+        <v/>
+      </c>
+      <c r="K71" s="28">
+        <f>IFERROR(K70/K69, "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="23" t="inlineStr">
+        <is>
+          <t>Actual Stage ΔV (verification)</t>
+        </is>
+      </c>
+      <c r="B72" s="24" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="E72" s="13">
+        <f>IFERROR(E33*9.80665*LN(E71), "")</f>
+        <v/>
+      </c>
+      <c r="H72" s="13">
+        <f>IFERROR(H33*9.80665*LN(H71), "")</f>
+        <v/>
+      </c>
+      <c r="K72" s="13">
+        <f>IFERROR(K33*9.80665*LN(K71), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>Thrust-to-Weight Ratio (at ignition)</t>
+        </is>
+      </c>
+      <c r="B73" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E73" s="29">
+        <f>IFERROR(E20*IFERROR(VLOOKUP(E19,'Engine DB'!$A:$K,7,0),0)*1000/(E70*9.80665), "")</f>
+        <v/>
+      </c>
+      <c r="H73" s="29">
+        <f>IFERROR(H20*IFERROR(VLOOKUP(H19,'Engine DB'!$A:$K,6,0),0)*1000/(H70*9.80665), "")</f>
+        <v/>
+      </c>
+      <c r="K73" s="29">
+        <f>IFERROR(K20*IFERROR(VLOOKUP(K19,'Engine DB'!$A:$K,6,0),0)*1000/(K70*9.80665), "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="inlineStr">
+        <is>
           <t>Propellant Mass Fraction</t>
         </is>
       </c>
-      <c r="B71" s="12" t="inlineStr">
+      <c r="B74" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E71" s="28">
-        <f>IFERROR(E22/E67, "")</f>
-        <v/>
-      </c>
-      <c r="H71" s="28">
-        <f>IFERROR(H22/H67, "")</f>
-        <v/>
-      </c>
-      <c r="K71" s="28">
-        <f>IFERROR(K22/K67, "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73" ht="18" customHeight="1">
-      <c r="A73" s="7" t="inlineStr">
+      <c r="E74" s="28">
+        <f>IFERROR(E24/E70, "")</f>
+        <v/>
+      </c>
+      <c r="H74" s="28">
+        <f>IFERROR(H24/H70, "")</f>
+        <v/>
+      </c>
+      <c r="K74" s="28">
+        <f>IFERROR(K24/K70, "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="7" t="inlineStr">
         <is>
           <t>VEHICLE SUMMARY</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="30" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="30" t="inlineStr">
         <is>
           <t>Max Payload to LEO</t>
         </is>
       </c>
-      <c r="B74" s="31">
-        <f>B61</f>
-        <v/>
-      </c>
-      <c r="C74" s="32" t="inlineStr">
+      <c r="B77" s="31">
+        <f>B64</f>
+        <v/>
+      </c>
+      <c r="C77" s="32" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="30" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="30" t="inlineStr">
         <is>
           <t>Max Payload to GTO</t>
         </is>
       </c>
-      <c r="B75" s="31">
-        <f>B64</f>
-        <v/>
-      </c>
-      <c r="C75" s="32" t="inlineStr">
+      <c r="B78" s="31">
+        <f>B67</f>
+        <v/>
+      </c>
+      <c r="C78" s="32" t="inlineStr">
         <is>
           <t>kg</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="33" t="inlineStr">
-        <is>
-          <t>LEO Payload Fraction (GLOW)</t>
-        </is>
-      </c>
-      <c r="B76" s="34">
-        <f>IFERROR(B61/E67*100, "")</f>
-        <v/>
-      </c>
-      <c r="C76" s="32" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="33" t="inlineStr">
-        <is>
-          <t>Total Vehicle ΔV (actual)</t>
-        </is>
-      </c>
-      <c r="B77" s="35">
-        <f>IFERROR(E69*1,0)+IFERROR(H69*1,0)+IFERROR(K69*1,0)</f>
-        <v/>
-      </c>
-      <c r="C77" s="32" t="inlineStr">
-        <is>
-          <t>m/s</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="33" t="inlineStr">
-        <is>
-          <t>LEO ΔV Margin vs Mission</t>
-        </is>
-      </c>
-      <c r="B78" s="35">
-        <f>IFERROR(E69*1,0)+IFERROR(H69*1,0)+IFERROR(K69*1,0)-B39</f>
-        <v/>
-      </c>
-      <c r="C78" s="32" t="inlineStr">
-        <is>
-          <t>m/s</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="33" t="inlineStr">
         <is>
-          <t>Gross Liftoff Mass (GLOW)</t>
-        </is>
-      </c>
-      <c r="B79" s="35">
-        <f>IFERROR(E67, "")</f>
+          <t>LEO Payload Fraction (GLOW)</t>
+        </is>
+      </c>
+      <c r="B79" s="34">
+        <f>IFERROR(B64/E70*100, "")</f>
         <v/>
       </c>
       <c r="C79" s="32" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>%</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="33" t="inlineStr">
         <is>
+          <t>Total Vehicle ΔV (actual)</t>
+        </is>
+      </c>
+      <c r="B80" s="35">
+        <f>IFERROR(E72*1,0)+IFERROR(H72*1,0)+IFERROR(K72*1,0)</f>
+        <v/>
+      </c>
+      <c r="C80" s="32" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="33" t="inlineStr">
+        <is>
+          <t>LEO ΔV Margin vs Mission</t>
+        </is>
+      </c>
+      <c r="B81" s="35">
+        <f>IFERROR(E72*1,0)+IFERROR(H72*1,0)+IFERROR(K72*1,0)-B42</f>
+        <v/>
+      </c>
+      <c r="C81" s="32" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="33" t="inlineStr">
+        <is>
+          <t>Gross Liftoff Mass (GLOW)</t>
+        </is>
+      </c>
+      <c r="B82" s="35">
+        <f>IFERROR(E70, "")</f>
+        <v/>
+      </c>
+      <c r="C82" s="32" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="33" t="inlineStr">
+        <is>
           <t>Total Propellant Mass</t>
         </is>
       </c>
-      <c r="B80" s="35">
-        <f>IFERROR(E22,0)+IFERROR(H22,0)+IFERROR(K22,0)</f>
-        <v/>
-      </c>
-      <c r="C80" s="32" t="inlineStr">
+      <c r="B83" s="35">
+        <f>IFERROR(E24,0)+IFERROR(H24,0)+IFERROR(K24,0)</f>
+        <v/>
+      </c>
+      <c r="C83" s="32" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="C61:L61"/>
+  <mergeCells count="23">
     <mergeCell ref="C8:L8"/>
-    <mergeCell ref="A15:K15"/>
-    <mergeCell ref="A73:K73"/>
-    <mergeCell ref="A60:K60"/>
+    <mergeCell ref="C67:L67"/>
     <mergeCell ref="C13:L13"/>
+    <mergeCell ref="C15:L15"/>
+    <mergeCell ref="A66:K66"/>
+    <mergeCell ref="A37:K37"/>
     <mergeCell ref="G3:H3"/>
+    <mergeCell ref="C14:L14"/>
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="C64:L64"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A47:K47"/>
+    <mergeCell ref="A76:K76"/>
     <mergeCell ref="C10:L10"/>
     <mergeCell ref="D3:E3"/>
-    <mergeCell ref="C41:L41"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="C44:L44"/>
     <mergeCell ref="J3:K3"/>
-    <mergeCell ref="A35:K35"/>
     <mergeCell ref="C9:L9"/>
     <mergeCell ref="A63:K63"/>
     <mergeCell ref="C12:L12"/>
-    <mergeCell ref="A44:K44"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="C11:L11"/>
   </mergeCells>
@@ -2112,7 +2159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A54"/>
+  <dimension ref="A1:A99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2462,6 +2509,289 @@
       <c r="A54" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">  Treat parallel-burn vehicles (Soyuz, Ariane 5) as series stages for delta-v calculation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="37" t="inlineStr"/>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="36" t="inlineStr">
+        <is>
+          <t>MAJOR SIMPLIFYING ASSUMPTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="37" t="inlineStr">
+        <is>
+          <t>The following assumptions are baked into this model. Understanding them helps interpret results:</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="16" customHeight="1">
+      <c r="A58" s="37" t="inlineStr"/>
+    </row>
+    <row r="59" ht="16" customHeight="1">
+      <c r="A59" s="37" t="inlineStr">
+        <is>
+          <t>1. GRAVITY LOSS MODEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="16" customHeight="1">
+      <c r="A60" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Gravity loss = (Gravity Loss Coefficient / TWR_liftoff) + Recovery Trajectory Penalty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="16" customHeight="1">
+      <c r="A61" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   The TWR term captures the effect of liftoff acceleration on the gravity turn. The trajectory</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="16" customHeight="1">
+      <c r="A62" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   penalty is an additive correction for the extra gravity loss incurred by recovery-optimized</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="16" customHeight="1">
+      <c r="A63" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   pitch profiles (shallower pitch angle = more time fighting gravity). Calibrate both inputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="16" customHeight="1">
+      <c r="A64" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   against a known vehicle. Typical total gravity loss: Expendable ~1,200–1,500 m/s (penalty=0);</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="16" customHeight="1">
+      <c r="A65" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ASDS ~1,700–2,000 m/s (penalty ~500 m/s); RTLS ~2,100–2,500 m/s (penalty ~900 m/s).</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="16" customHeight="1">
+      <c r="A66" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Remaining limitation: the model still cannot distinguish trajectory shape within a mission class</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="16" customHeight="1">
+      <c r="A67" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   (e.g. a high-TWR expendable vs a low-TWR expendable will have the same penalty).</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="16" customHeight="1">
+      <c r="A68" s="37" t="inlineStr"/>
+    </row>
+    <row r="69" ht="16" customHeight="1">
+      <c r="A69" s="37" t="inlineStr">
+        <is>
+          <t>2. EFFECTIVE ISP IS A LINEAR ATMOSPHERIC BLEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="16" customHeight="1">
+      <c r="A70" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Isp_eff = Isp_SL + Atm_Fraction × (Isp_vac - Isp_SL). The Atm Fraction input is a scalar</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="16" customHeight="1">
+      <c r="A71" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   approximation of what is actually a continuous altitude-pressure curve. For sea-level-optimized</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="16" customHeight="1">
+      <c r="A72" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   nozzles this can be off by 5–10 s depending on the vehicle's ascent profile. Default: 0.6 for S1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="16" customHeight="1">
+      <c r="A73" s="37" t="inlineStr"/>
+    </row>
+    <row r="74" ht="16" customHeight="1">
+      <c r="A74" s="37" t="inlineStr">
+        <is>
+          <t>3. GLOW INCLUDES PAYLOAD (ITERATIVE — see note below)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="16" customHeight="1">
+      <c r="A75" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   GLOW includes the solved payload mass so TWR and gravity loss are self-consistent. This creates</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="16" customHeight="1">
+      <c r="A76" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   a circular reference resolved by Excel's iterative calculation (File → Options → Formulas →</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="16" customHeight="1">
+      <c r="A77" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Enable iterative calculation). The workbook is saved with iteration enabled. If you see a</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="16" customHeight="1">
+      <c r="A78" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   circular reference error, ensure iterative calculation is turned on in your Excel settings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="16" customHeight="1">
+      <c r="A79" s="37" t="inlineStr"/>
+    </row>
+    <row r="80" ht="16" customHeight="1">
+      <c r="A80" s="37" t="inlineStr">
+        <is>
+          <t>4. RECOVERY IS MODELED AS A SINGLE BURN FROM DRY MASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="16" customHeight="1">
+      <c r="A81" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Recovery Propellant = eff_dry × (e^(ΔV_recovery / Isp / g₀) - 1). Real recovery sequences</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="16" customHeight="1">
+      <c r="A82" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   have multiple burns (entry burn from partially-fueled stage, landing burn from near-dry stage),</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="16" customHeight="1">
+      <c r="A83" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   each starting from different initial masses. A single-burn model slightly underestimates total</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="16" customHeight="1">
+      <c r="A84" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   recovery propellant. The error is typically 5–15% of recovery propellant (~1–3% of total prop).</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="16" customHeight="1">
+      <c r="A85" s="37" t="inlineStr"/>
+    </row>
+    <row r="86" ht="16" customHeight="1">
+      <c r="A86" s="37" t="inlineStr">
+        <is>
+          <t>5. FAIRING MASS IS NOT EXPLICITLY MODELED</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="16" customHeight="1">
+      <c r="A87" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   The payload fairing (typically 1,700–2,000 kg for a 5m fairing) is jettisoned mid-ascent during</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="16" customHeight="1">
+      <c r="A88" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   S1 burn. This model does not account for fairing jettison as a discrete mass event. In practice,</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="16" customHeight="1">
+      <c r="A89" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   fairing mass is often included in the reported payload adapter mass as a workaround.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="16" customHeight="1">
+      <c r="A90" s="37" t="inlineStr"/>
+    </row>
+    <row r="91" ht="16" customHeight="1">
+      <c r="A91" s="37" t="inlineStr">
+        <is>
+          <t>6. GTO ΔV IS A FIXED INPUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="16" customHeight="1">
+      <c r="A92" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   The GTO Orbital ΔV input (default 10,400 m/s) does not vary with launch site latitude, target</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="16" customHeight="1">
+      <c r="A93" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   inclination, apogee altitude, or insertion strategy. GTO missions vary by 300–600 m/s depending</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="16" customHeight="1">
+      <c r="A94" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   on these parameters. Tune this value for specific mission comparisons.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="16" customHeight="1">
+      <c r="A95" s="37" t="inlineStr"/>
+    </row>
+    <row r="96" ht="16" customHeight="1">
+      <c r="A96" s="37" t="inlineStr">
+        <is>
+          <t>7. ISP DOES NOT VARY WITH THROTTLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="16" customHeight="1">
+      <c r="A97" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Engines are modeled at a fixed Isp. In reality, throttling changes chamber pressure and mixture</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="16" customHeight="1">
+      <c r="A98" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ratio, shifting Isp by ~1–3%. This matters most for engines that throttle deeply (Merlin 1D</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="16" customHeight="1">
+      <c r="A99" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   throttles to ~40% for landing burns). Effect on ascent performance is small but non-zero.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
gravity loss model was getting more complicated that we can justify or support with meaningful numbers.
</commit_message>
<xml_diff>
--- a/launch_vehicle_design.xlsx
+++ b/launch_vehicle_design.xlsx
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M83"/>
+  <dimension ref="A1:M81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -877,14 +877,14 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>← Base gravity loss = coeff / TWR_liftoff (trajectory-independent term); ~1750 typical</t>
+          <t>← Base gravity loss = coeff / TWR_liftoff; ~1750 typical for expendable; increase to match reusable vehicles</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>LEO Trajectory Penalty</t>
+          <t>Trajectory Penalty</t>
         </is>
       </c>
       <c r="B12" s="10" t="n">
@@ -892,81 +892,89 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>← Extra gravity loss for LEO recovery pitch profile; 0=expendable, ~500=ASDS, ~900=RTLS</t>
+          <t>← Additive gravity loss for recovery pitch profile; 0=expendable, calibrate to match known vehicle — default 500 m/s for F9 ASDS</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>GTO Trajectory Penalty</t>
+          <t>GTO Orbital ΔV</t>
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>100</v>
+        <v>10400</v>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>← Extra gravity loss for GTO pitch profile; smaller than LEO — S1 burns less time/downrange; ~0-150 m/s typical</t>
+          <t>← Velocity needed at GTO perigee — ~10,200-10,500 m/s depending on inclination and target apogee</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>GTO Orbital ΔV</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n">
-        <v>10400</v>
+          <t>Number of Stages</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>2</v>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>← Velocity needed at GTO perigee — ~10,200-10,500 m/s depending on inclination and target apogee</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Number of Stages</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
           <t>← Active stages (enter 1-3)</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>STAGE CONFIGURATION</t>
         </is>
       </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Stage Name</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>S1 Core</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>S2 Upper</t>
+        </is>
+      </c>
+      <c r="K17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Stage Name</t>
+          <t>Engine (from Engine DB)</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>name</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>S1 Core</t>
+          <t>Merlin 1D</t>
         </is>
       </c>
       <c r="H18" s="9" t="inlineStr">
         <is>
-          <t>S2 Upper</t>
+          <t>Merlin 1D Vac</t>
         </is>
       </c>
       <c r="K18" s="9" t="inlineStr"/>
@@ -974,224 +982,216 @@
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Engine (from Engine DB)</t>
+          <t>Number of Engines</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>Merlin 1D</t>
-        </is>
-      </c>
-      <c r="H19" s="9" t="inlineStr">
-        <is>
-          <t>Merlin 1D Vac</t>
-        </is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="H19" s="9" t="n">
+        <v>1</v>
       </c>
       <c r="K19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Number of Engines</t>
+          <t>Propellant Combination</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>count</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>1</v>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>LOX/RP-1</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>LOX/RP-1</t>
+        </is>
       </c>
       <c r="K20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Propellant Combination</t>
+          <t>Propellant Mass (nominal)</t>
         </is>
       </c>
       <c r="B21" s="12" t="inlineStr">
         <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>LOX/RP-1</t>
-        </is>
-      </c>
-      <c r="H21" s="9" t="inlineStr">
-        <is>
-          <t>LOX/RP-1</t>
-        </is>
-      </c>
-      <c r="K21" s="9" t="inlineStr"/>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E21" s="10" t="n">
+        <v>411000</v>
+      </c>
+      <c r="H21" s="10" t="n">
+        <v>111500</v>
+      </c>
+      <c r="K21" s="10" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Propellant Mass (nominal)</t>
+          <t>Subcooling Gain (%)</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E22" s="10" t="n">
-        <v>411000</v>
-      </c>
-      <c r="H22" s="10" t="n">
-        <v>111500</v>
-      </c>
-      <c r="K22" s="10" t="inlineStr"/>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K22" s="9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Subcooling Gain (%)</t>
+          <t>Effective Propellant Mass</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="9" t="n">
-        <v>0</v>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E23" s="13">
+        <f>IFERROR(E21*(1+E22/100),"")</f>
+        <v/>
+      </c>
+      <c r="H23" s="13">
+        <f>IFERROR(H21*(1+H22/100),"")</f>
+        <v/>
+      </c>
+      <c r="K23" s="13">
+        <f>IFERROR(K21*(1+K22/100),"")</f>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>Effective Propellant Mass</t>
+          <t>Recovery ΔV Reserve (m/s)</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E24" s="13">
-        <f>IFERROR(E22*(1+E23/100),"")</f>
-        <v/>
-      </c>
-      <c r="H24" s="13">
-        <f>IFERROR(H22*(1+H23/100),"")</f>
-        <v/>
-      </c>
-      <c r="K24" s="13">
-        <f>IFERROR(K22*(1+K23/100),"")</f>
-        <v/>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="n">
+        <v>500</v>
+      </c>
+      <c r="H24" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Recovery ΔV Reserve (m/s)</t>
+          <t>Recovery Propellant Reserved</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>m/s</t>
-        </is>
-      </c>
-      <c r="E25" s="10" t="n">
-        <v>500</v>
-      </c>
-      <c r="H25" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" s="10" t="n">
-        <v>0</v>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E25" s="14">
+        <f>IFERROR(IF(E24=0,0,E59*(EXP(E24/(E29*9.80665))-1)),0)</f>
+        <v/>
+      </c>
+      <c r="H25" s="14">
+        <f>IFERROR(IF(H24=0,0,H59*(EXP(H24/(H29*9.80665))-1)),0)</f>
+        <v/>
+      </c>
+      <c r="K25" s="14">
+        <f>IFERROR(IF(K24=0,0,K59*(EXP(K24/(K29*9.80665))-1)),0)</f>
+        <v/>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>Recovery Propellant Reserved</t>
+          <t>LEO ΔV Fraction</t>
         </is>
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E26" s="14">
-        <f>IFERROR(IF(E25=0,0,E61*(EXP(E25/(E30*9.80665))-1)),0)</f>
-        <v/>
-      </c>
-      <c r="H26" s="14">
-        <f>IFERROR(IF(H25=0,0,H61*(EXP(H25/(H30*9.80665))-1)),0)</f>
-        <v/>
-      </c>
-      <c r="K26" s="14">
-        <f>IFERROR(IF(K25=0,0,K61*(EXP(K25/(K30*9.80665))-1)),0)</f>
-        <v/>
-      </c>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="K26" s="9" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>LEO ΔV Fraction</t>
+          <t>LEO ΔV Allocation</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>0-1</t>
-        </is>
-      </c>
-      <c r="E27" s="9" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H27" s="9" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="K27" s="9" t="inlineStr"/>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="E27" s="14">
+        <f>IFERROR(E26*B40,"")</f>
+        <v/>
+      </c>
+      <c r="H27" s="14">
+        <f>IFERROR(H26*B40,"")</f>
+        <v/>
+      </c>
+      <c r="K27" s="14">
+        <f>IFERROR(K26*B40,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>LEO ΔV Allocation</t>
+          <t>Vac Isp Override</t>
         </is>
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>m/s</t>
-        </is>
-      </c>
-      <c r="E28" s="14">
-        <f>IFERROR(E27*B42,"")</f>
-        <v/>
-      </c>
-      <c r="H28" s="14">
-        <f>IFERROR(H27*B42,"")</f>
-        <v/>
-      </c>
-      <c r="K28" s="14">
-        <f>IFERROR(K27*B42,"")</f>
-        <v/>
-      </c>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr"/>
+      <c r="H28" s="9" t="inlineStr"/>
+      <c r="K28" s="9" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Vac Isp Override</t>
+          <t>Vac Isp (from DB)</t>
         </is>
       </c>
       <c r="B29" s="12" t="inlineStr">
@@ -1199,14 +1199,23 @@
           <t>s</t>
         </is>
       </c>
-      <c r="E29" s="9" t="inlineStr"/>
-      <c r="H29" s="9" t="inlineStr"/>
-      <c r="K29" s="9" t="inlineStr"/>
+      <c r="E29" s="15">
+        <f>IF(E28&lt;&gt;"",E28,IFERROR(VLOOKUP(E18,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+        <v/>
+      </c>
+      <c r="H29" s="15">
+        <f>IF(H28&lt;&gt;"",H28,IFERROR(VLOOKUP(H18,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+        <v/>
+      </c>
+      <c r="K29" s="15">
+        <f>IF(K28&lt;&gt;"",K28,IFERROR(VLOOKUP(K18,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Vac Isp (from DB)</t>
+          <t>SL Isp (from DB)</t>
         </is>
       </c>
       <c r="B30" s="12" t="inlineStr">
@@ -1215,253 +1224,266 @@
         </is>
       </c>
       <c r="E30" s="15">
-        <f>IF(E29&lt;&gt;"",E29,IFERROR(VLOOKUP(E19,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+        <f>IFERROR(VLOOKUP(E18,'Engine DB'!$A:$K,5,0),"—")</f>
         <v/>
       </c>
       <c r="H30" s="15">
-        <f>IF(H29&lt;&gt;"",H29,IFERROR(VLOOKUP(H19,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+        <f>IFERROR(VLOOKUP(H18,'Engine DB'!$A:$K,5,0),"—")</f>
         <v/>
       </c>
       <c r="K30" s="15">
-        <f>IF(K29&lt;&gt;"",K29,IFERROR(VLOOKUP(K19,'Engine DB'!$A:$K,4,0),"Enter engine"))</f>
+        <f>IFERROR(VLOOKUP(K18,'Engine DB'!$A:$K,5,0),"—")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>SL Isp (from DB)</t>
+          <t>Atm Fraction (0-1)</t>
         </is>
       </c>
       <c r="B31" s="12" t="inlineStr">
         <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="E31" s="15">
-        <f>IFERROR(VLOOKUP(E19,'Engine DB'!$A:$K,5,0),"—")</f>
-        <v/>
-      </c>
-      <c r="H31" s="15">
-        <f>IFERROR(VLOOKUP(H19,'Engine DB'!$A:$K,5,0),"—")</f>
-        <v/>
-      </c>
-      <c r="K31" s="15">
-        <f>IFERROR(VLOOKUP(K19,'Engine DB'!$A:$K,5,0),"—")</f>
-        <v/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H31" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K31" s="9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>Atm Fraction (0-1)</t>
+          <t>Effective Isp (used)</t>
         </is>
       </c>
       <c r="B32" s="12" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="H32" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="K32" s="9" t="n">
-        <v>1</v>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E32" s="16">
+        <f>IFERROR(IF(ISNUMBER(E30),E30+E31*(E29-E30),E29),E29)</f>
+        <v/>
+      </c>
+      <c r="H32" s="16">
+        <f>IFERROR(IF(ISNUMBER(H30),H30+H31*(H29-H30),H29),H29)</f>
+        <v/>
+      </c>
+      <c r="K32" s="16">
+        <f>IFERROR(IF(ISNUMBER(K30),K30+K31*(K29-K30),K29),K29)</f>
+        <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>Effective Isp (used)</t>
+          <t>GTO ΔV Fraction</t>
         </is>
       </c>
       <c r="B33" s="12" t="inlineStr">
         <is>
-          <t>s</t>
-        </is>
-      </c>
-      <c r="E33" s="16">
-        <f>IFERROR(IF(ISNUMBER(E31),E31+E32*(E30-E31),E30),E30)</f>
-        <v/>
-      </c>
-      <c r="H33" s="16">
-        <f>IFERROR(IF(ISNUMBER(H31),H31+H32*(H30-H31),H30),H30)</f>
-        <v/>
-      </c>
-      <c r="K33" s="16">
-        <f>IFERROR(IF(ISNUMBER(K31),K31+K32*(K30-K31),K30),K30)</f>
-        <v/>
-      </c>
+          <t>0-1</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="H33" s="9" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="K33" s="9" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>GTO ΔV Fraction</t>
+          <t>GTO ΔV Allocation</t>
         </is>
       </c>
       <c r="B34" s="12" t="inlineStr">
         <is>
-          <t>0-1</t>
-        </is>
-      </c>
-      <c r="E34" s="9" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="H34" s="9" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="K34" s="9" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>GTO ΔV Allocation</t>
-        </is>
-      </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
           <t>m/s</t>
         </is>
       </c>
-      <c r="E35" s="14">
-        <f>IFERROR(E34*B43,"")</f>
-        <v/>
-      </c>
-      <c r="H35" s="14">
-        <f>IFERROR(H34*B43,"")</f>
-        <v/>
-      </c>
-      <c r="K35" s="14">
-        <f>IFERROR(K34*B43,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="7" t="inlineStr">
+      <c r="E34" s="14">
+        <f>IFERROR(E33*B41,"")</f>
+        <v/>
+      </c>
+      <c r="H34" s="14">
+        <f>IFERROR(H33*B41,"")</f>
+        <v/>
+      </c>
+      <c r="K34" s="14">
+        <f>IFERROR(K33*B41,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>MISSION ΔV ANALYSIS  —  Gravity loss computed from liftoff TWR</t>
         </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>Est. GLOW (stage masses only, no payload)</t>
+        </is>
+      </c>
+      <c r="B37" s="14">
+        <f>IFERROR(E21+E59,0)+IFERROR(H21+H59,0)+IFERROR(K21+K59,0)</f>
+        <v/>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>Est. GLOW (stage masses only, no payload)</t>
-        </is>
-      </c>
-      <c r="B38" s="14">
-        <f>IFERROR(E22+E61,0)+IFERROR(H22+H61,0)+IFERROR(K22+K61,0)</f>
+          <t>Stage 1 Liftoff TWR (est., no payload)</t>
+        </is>
+      </c>
+      <c r="B38" s="17">
+        <f>IFERROR(E19*IFERROR(VLOOKUP(E18,'Engine DB'!$A:$K,7,0),0)*1000/(B37*9.80665),"")</f>
         <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
         <is>
-          <t>Stage 1 Liftoff TWR (est., no payload)</t>
-        </is>
-      </c>
-      <c r="B39" s="17">
-        <f>IFERROR(E20*IFERROR(VLOOKUP(E19,'Engine DB'!$A:$K,7,0),0)*1000/(B38*9.80665),"")</f>
+          <t>Gravity Loss (= coeff / TWR + trajectory penalty)</t>
+        </is>
+      </c>
+      <c r="B39" s="14">
+        <f>IFERROR(B11/B38+B12,"")</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>LEO Gravity Loss (= coeff / TWR + LEO penalty)</t>
-        </is>
-      </c>
-      <c r="B40" s="14">
-        <f>IFERROR(B11/B39+B12,"")</f>
+          <t>LEO Mission ΔV (calculated)</t>
+        </is>
+      </c>
+      <c r="B40" s="18">
+        <f>IFERROR(B9+B10+B39,"")</f>
         <v/>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>GTO Gravity Loss (= coeff / TWR + GTO penalty)</t>
-        </is>
-      </c>
-      <c r="B41" s="14">
-        <f>IFERROR(B11/B39+B13,"")</f>
+          <t>GTO Mission ΔV (calculated)</t>
+        </is>
+      </c>
+      <c r="B41" s="18">
+        <f>IFERROR(B13+B10+B39,"")</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t>LEO Mission ΔV (calculated)</t>
-        </is>
-      </c>
-      <c r="B42" s="18">
-        <f>IFERROR(B9+B10+B40,"")</f>
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>LEO ΔV Allocation Check (should = LEO Mission ΔV above)</t>
+        </is>
+      </c>
+      <c r="B42" s="20">
+        <f>IFERROR(E27*1,0)+IFERROR(H27*1,0)+IFERROR(K27*1,0)</f>
+        <v/>
+      </c>
+      <c r="C42" s="2">
+        <f>IF(ABS(B42-B40)&lt;1,"✓ OK","⚠ Adjust stage allocations to sum to LEO Mission ΔV")</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>GTO Mission ΔV (calculated)</t>
-        </is>
-      </c>
-      <c r="B43" s="18">
-        <f>IFERROR(B14+B10+B41,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="19" t="inlineStr">
-        <is>
-          <t>LEO ΔV Allocation Check (should = LEO Mission ΔV above)</t>
-        </is>
-      </c>
-      <c r="B44" s="20">
-        <f>IFERROR(E28*1,0)+IFERROR(H28*1,0)+IFERROR(K28*1,0)</f>
-        <v/>
-      </c>
-      <c r="C44" s="2">
-        <f>IF(ABS(B44-B42)&lt;1,"✓ OK","⚠ Adjust stage allocations to sum to LEO Mission ΔV")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
           <t>Engine Mass per Engine</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B43" s="12" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E45" s="21">
-        <f>IFERROR(VLOOKUP(E19,'Engine DB'!$A:$K,8,0),"—")</f>
-        <v/>
-      </c>
-      <c r="H45" s="21">
-        <f>IFERROR(VLOOKUP(H19,'Engine DB'!$A:$K,8,0),"—")</f>
-        <v/>
-      </c>
-      <c r="K45" s="21">
-        <f>IFERROR(VLOOKUP(K19,'Engine DB'!$A:$K,8,0),"—")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="7" t="inlineStr">
+      <c r="E43" s="21">
+        <f>IFERROR(VLOOKUP(E18,'Engine DB'!$A:$K,8,0),"—")</f>
+        <v/>
+      </c>
+      <c r="H43" s="21">
+        <f>IFERROR(VLOOKUP(H18,'Engine DB'!$A:$K,8,0),"—")</f>
+        <v/>
+      </c>
+      <c r="K43" s="21">
+        <f>IFERROR(VLOOKUP(K18,'Engine DB'!$A:$K,8,0),"—")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
         <is>
           <t>SUBSYSTEM MASS BREAKDOWN (auto-estimated; override any yellow cell)</t>
         </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="22" t="inlineStr">
+        <is>
+          <t>Tank Structure</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E46" s="10">
+        <f>IF(E21="","",E21/100*IF(E20="LOX/RP-1",3.5,IF(E20="LOX/LH2",6.5,IF(E20="LOX/CH4",3.8,IF(OR(E20="Solid HTPB",E20="Solid PBAN"),1.8,2.5)))))</f>
+        <v/>
+      </c>
+      <c r="H46" s="10">
+        <f>IF(H21="","",H21/100*IF(H20="LOX/RP-1",3.5,IF(H20="LOX/LH2",6.5,IF(H20="LOX/CH4",3.8,IF(OR(H20="Solid HTPB",H20="Solid PBAN"),1.8,2.5)))))</f>
+        <v/>
+      </c>
+      <c r="K46" s="10">
+        <f>IF(K21="","",K21/100*IF(K20="LOX/RP-1",3.5,IF(K20="LOX/LH2",6.5,IF(K20="LOX/CH4",3.8,IF(OR(K20="Solid HTPB",K20="Solid PBAN"),1.8,2.5)))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="22" t="inlineStr">
+        <is>
+          <t>Pressurization System</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E47" s="10">
+        <f>IF(E21="","",E21/100*IF(E20="LOX/RP-1",0.4,IF(E20="LOX/LH2",0.6,IF(E20="LOX/CH4",0.4,IF(OR(E20="Solid HTPB",E20="Solid PBAN"),0.0,0.5)))))</f>
+        <v/>
+      </c>
+      <c r="H47" s="10">
+        <f>IF(H21="","",H21/100*IF(H20="LOX/RP-1",0.4,IF(H20="LOX/LH2",0.6,IF(H20="LOX/CH4",0.4,IF(OR(H20="Solid HTPB",H20="Solid PBAN"),0.0,0.5)))))</f>
+        <v/>
+      </c>
+      <c r="K47" s="10">
+        <f>IF(K21="","",K21/100*IF(K20="LOX/RP-1",0.4,IF(K20="LOX/LH2",0.6,IF(K20="LOX/CH4",0.4,IF(OR(K20="Solid HTPB",K20="Solid PBAN"),0.0,0.5)))))</f>
+        <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="22" t="inlineStr">
         <is>
-          <t>Tank Structure</t>
+          <t>Feed System / Plumbing</t>
         </is>
       </c>
       <c r="B48" s="12" t="inlineStr">
@@ -1470,22 +1492,22 @@
         </is>
       </c>
       <c r="E48" s="10">
-        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",3.5,IF(E21="LOX/LH2",6.5,IF(E21="LOX/CH4",3.8,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),1.8,2.5)))))</f>
+        <f>IF(E21="","",E21/100*IF(E20="LOX/RP-1",0.8,IF(E20="LOX/LH2",1.0,IF(E20="LOX/CH4",0.8,IF(OR(E20="Solid HTPB",E20="Solid PBAN"),0.2,0.6)))))</f>
         <v/>
       </c>
       <c r="H48" s="10">
-        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",3.5,IF(H21="LOX/LH2",6.5,IF(H21="LOX/CH4",3.8,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),1.8,2.5)))))</f>
+        <f>IF(H21="","",H21/100*IF(H20="LOX/RP-1",0.8,IF(H20="LOX/LH2",1.0,IF(H20="LOX/CH4",0.8,IF(OR(H20="Solid HTPB",H20="Solid PBAN"),0.2,0.6)))))</f>
         <v/>
       </c>
       <c r="K48" s="10">
-        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",3.5,IF(K21="LOX/LH2",6.5,IF(K21="LOX/CH4",3.8,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),1.8,2.5)))))</f>
+        <f>IF(K21="","",K21/100*IF(K20="LOX/RP-1",0.8,IF(K20="LOX/LH2",1.0,IF(K20="LOX/CH4",0.8,IF(OR(K20="Solid HTPB",K20="Solid PBAN"),0.2,0.6)))))</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="22" t="inlineStr">
         <is>
-          <t>Pressurization System</t>
+          <t>Avionics / GNC</t>
         </is>
       </c>
       <c r="B49" s="12" t="inlineStr">
@@ -1494,22 +1516,22 @@
         </is>
       </c>
       <c r="E49" s="10">
-        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.4,IF(E21="LOX/LH2",0.6,IF(E21="LOX/CH4",0.4,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.0,0.5)))))</f>
+        <f>IF(E21="","",E21/100*IF(E20="LOX/RP-1",0.3,IF(E20="LOX/LH2",0.4,IF(E20="LOX/CH4",0.3,IF(OR(E20="Solid HTPB",E20="Solid PBAN"),0.2,0.4)))))</f>
         <v/>
       </c>
       <c r="H49" s="10">
-        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.4,IF(H21="LOX/LH2",0.6,IF(H21="LOX/CH4",0.4,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.0,0.5)))))</f>
+        <f>IF(H21="","",H21/100*IF(H20="LOX/RP-1",0.3,IF(H20="LOX/LH2",0.4,IF(H20="LOX/CH4",0.3,IF(OR(H20="Solid HTPB",H20="Solid PBAN"),0.2,0.4)))))</f>
         <v/>
       </c>
       <c r="K49" s="10">
-        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.4,IF(K21="LOX/LH2",0.6,IF(K21="LOX/CH4",0.4,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.0,0.5)))))</f>
+        <f>IF(K21="","",K21/100*IF(K20="LOX/RP-1",0.3,IF(K20="LOX/LH2",0.4,IF(K20="LOX/CH4",0.3,IF(OR(K20="Solid HTPB",K20="Solid PBAN"),0.2,0.4)))))</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="22" t="inlineStr">
         <is>
-          <t>Feed System / Plumbing</t>
+          <t>Power System</t>
         </is>
       </c>
       <c r="B50" s="12" t="inlineStr">
@@ -1518,22 +1540,22 @@
         </is>
       </c>
       <c r="E50" s="10">
-        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.8,IF(E21="LOX/LH2",1.0,IF(E21="LOX/CH4",0.8,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.2,0.6)))))</f>
+        <f>IF(E21="","",E21/100*IF(E20="LOX/RP-1",0.2,IF(E20="LOX/LH2",0.3,IF(E20="LOX/CH4",0.2,IF(OR(E20="Solid HTPB",E20="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
       <c r="H50" s="10">
-        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.8,IF(H21="LOX/LH2",1.0,IF(H21="LOX/CH4",0.8,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.2,0.6)))))</f>
+        <f>IF(H21="","",H21/100*IF(H20="LOX/RP-1",0.2,IF(H20="LOX/LH2",0.3,IF(H20="LOX/CH4",0.2,IF(OR(H20="Solid HTPB",H20="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
       <c r="K50" s="10">
-        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.8,IF(K21="LOX/LH2",1.0,IF(K21="LOX/CH4",0.8,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.2,0.6)))))</f>
+        <f>IF(K21="","",K21/100*IF(K20="LOX/RP-1",0.2,IF(K20="LOX/LH2",0.3,IF(K20="LOX/CH4",0.2,IF(OR(K20="Solid HTPB",K20="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="22" t="inlineStr">
         <is>
-          <t>Avionics / GNC</t>
+          <t>Thermal Control</t>
         </is>
       </c>
       <c r="B51" s="12" t="inlineStr">
@@ -1542,22 +1564,22 @@
         </is>
       </c>
       <c r="E51" s="10">
-        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.3,IF(E21="LOX/LH2",0.4,IF(E21="LOX/CH4",0.3,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.2,0.4)))))</f>
+        <f>IF(E21="","",E21/100*IF(E20="LOX/RP-1",0.2,IF(E20="LOX/LH2",1.0,IF(E20="LOX/CH4",0.3,IF(OR(E20="Solid HTPB",E20="Solid PBAN"),0.1,0.3)))))</f>
         <v/>
       </c>
       <c r="H51" s="10">
-        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.3,IF(H21="LOX/LH2",0.4,IF(H21="LOX/CH4",0.3,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.2,0.4)))))</f>
+        <f>IF(H21="","",H21/100*IF(H20="LOX/RP-1",0.2,IF(H20="LOX/LH2",1.0,IF(H20="LOX/CH4",0.3,IF(OR(H20="Solid HTPB",H20="Solid PBAN"),0.1,0.3)))))</f>
         <v/>
       </c>
       <c r="K51" s="10">
-        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.3,IF(K21="LOX/LH2",0.4,IF(K21="LOX/CH4",0.3,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.2,0.4)))))</f>
+        <f>IF(K21="","",K21/100*IF(K20="LOX/RP-1",0.2,IF(K20="LOX/LH2",1.0,IF(K20="LOX/CH4",0.3,IF(OR(K20="Solid HTPB",K20="Solid PBAN"),0.1,0.3)))))</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="22" t="inlineStr">
         <is>
-          <t>Power System</t>
+          <t>RCS / ACS</t>
         </is>
       </c>
       <c r="B52" s="12" t="inlineStr">
@@ -1566,22 +1588,22 @@
         </is>
       </c>
       <c r="E52" s="10">
-        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.2,IF(E21="LOX/LH2",0.3,IF(E21="LOX/CH4",0.2,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(E21="","",E21/100*IF(E20="LOX/RP-1",0.3,IF(E20="LOX/LH2",0.4,IF(E20="LOX/CH4",0.3,IF(OR(E20="Solid HTPB",E20="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
       <c r="H52" s="10">
-        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.2,IF(H21="LOX/LH2",0.3,IF(H21="LOX/CH4",0.2,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(H21="","",H21/100*IF(H20="LOX/RP-1",0.3,IF(H20="LOX/LH2",0.4,IF(H20="LOX/CH4",0.3,IF(OR(H20="Solid HTPB",H20="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
       <c r="K52" s="10">
-        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.2,IF(K21="LOX/LH2",0.3,IF(K21="LOX/CH4",0.2,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(K21="","",K21/100*IF(K20="LOX/RP-1",0.3,IF(K20="LOX/LH2",0.4,IF(K20="LOX/CH4",0.3,IF(OR(K20="Solid HTPB",K20="Solid PBAN"),0.1,0.2)))))</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="22" t="inlineStr">
         <is>
-          <t>Thermal Control</t>
+          <t>Separation System</t>
         </is>
       </c>
       <c r="B53" s="12" t="inlineStr">
@@ -1590,22 +1612,22 @@
         </is>
       </c>
       <c r="E53" s="10">
-        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.2,IF(E21="LOX/LH2",1.0,IF(E21="LOX/CH4",0.3,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.1,0.3)))))</f>
+        <f>IF(E21="","",E21/100*IF(E20="LOX/RP-1",0.1,IF(E20="LOX/LH2",0.1,IF(E20="LOX/CH4",0.1,IF(OR(E20="Solid HTPB",E20="Solid PBAN"),0.1,0.1)))))</f>
         <v/>
       </c>
       <c r="H53" s="10">
-        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.2,IF(H21="LOX/LH2",1.0,IF(H21="LOX/CH4",0.3,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.1,0.3)))))</f>
+        <f>IF(H21="","",H21/100*IF(H20="LOX/RP-1",0.1,IF(H20="LOX/LH2",0.1,IF(H20="LOX/CH4",0.1,IF(OR(H20="Solid HTPB",H20="Solid PBAN"),0.1,0.1)))))</f>
         <v/>
       </c>
       <c r="K53" s="10">
-        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.2,IF(K21="LOX/LH2",1.0,IF(K21="LOX/CH4",0.3,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.1,0.3)))))</f>
+        <f>IF(K21="","",K21/100*IF(K20="LOX/RP-1",0.1,IF(K20="LOX/LH2",0.1,IF(K20="LOX/CH4",0.1,IF(OR(K20="Solid HTPB",K20="Solid PBAN"),0.1,0.1)))))</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="22" t="inlineStr">
         <is>
-          <t>RCS / ACS</t>
+          <t>Recovery Hardware</t>
         </is>
       </c>
       <c r="B54" s="12" t="inlineStr">
@@ -1614,22 +1636,22 @@
         </is>
       </c>
       <c r="E54" s="10">
-        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.3,IF(E21="LOX/LH2",0.4,IF(E21="LOX/CH4",0.3,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(E21="","",E21/100*IF(E20="LOX/RP-1",0.0,IF(E20="LOX/LH2",0.0,IF(E20="LOX/CH4",0.0,IF(OR(E20="Solid HTPB",E20="Solid PBAN"),0.0,0.0)))))</f>
         <v/>
       </c>
       <c r="H54" s="10">
-        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.3,IF(H21="LOX/LH2",0.4,IF(H21="LOX/CH4",0.3,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(H21="","",H21/100*IF(H20="LOX/RP-1",0.0,IF(H20="LOX/LH2",0.0,IF(H20="LOX/CH4",0.0,IF(OR(H20="Solid HTPB",H20="Solid PBAN"),0.0,0.0)))))</f>
         <v/>
       </c>
       <c r="K54" s="10">
-        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.3,IF(K21="LOX/LH2",0.4,IF(K21="LOX/CH4",0.3,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.1,0.2)))))</f>
+        <f>IF(K21="","",K21/100*IF(K20="LOX/RP-1",0.0,IF(K20="LOX/LH2",0.0,IF(K20="LOX/CH4",0.0,IF(OR(K20="Solid HTPB",K20="Solid PBAN"),0.0,0.0)))))</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="22" t="inlineStr">
         <is>
-          <t>Separation System</t>
+          <t>Residuals / Margin</t>
         </is>
       </c>
       <c r="B55" s="12" t="inlineStr">
@@ -1638,22 +1660,22 @@
         </is>
       </c>
       <c r="E55" s="10">
-        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.1,IF(E21="LOX/LH2",0.1,IF(E21="LOX/CH4",0.1,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.1,0.1)))))</f>
+        <f>IF(E21="","",E21/100*IF(E20="LOX/RP-1",0.5,IF(E20="LOX/LH2",0.8,IF(E20="LOX/CH4",0.5,IF(OR(E20="Solid HTPB",E20="Solid PBAN"),0.3,0.5)))))</f>
         <v/>
       </c>
       <c r="H55" s="10">
-        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.1,IF(H21="LOX/LH2",0.1,IF(H21="LOX/CH4",0.1,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.1,0.1)))))</f>
+        <f>IF(H21="","",H21/100*IF(H20="LOX/RP-1",0.5,IF(H20="LOX/LH2",0.8,IF(H20="LOX/CH4",0.5,IF(OR(H20="Solid HTPB",H20="Solid PBAN"),0.3,0.5)))))</f>
         <v/>
       </c>
       <c r="K55" s="10">
-        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.1,IF(K21="LOX/LH2",0.1,IF(K21="LOX/CH4",0.1,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.1,0.1)))))</f>
+        <f>IF(K21="","",K21/100*IF(K20="LOX/RP-1",0.5,IF(K20="LOX/LH2",0.8,IF(K20="LOX/CH4",0.5,IF(OR(K20="Solid HTPB",K20="Solid PBAN"),0.3,0.5)))))</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="22" t="inlineStr">
         <is>
-          <t>Recovery Hardware</t>
+          <t>Engine System Total</t>
         </is>
       </c>
       <c r="B56" s="12" t="inlineStr">
@@ -1661,47 +1683,47 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E56" s="10">
-        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.0,IF(E21="LOX/LH2",0.0,IF(E21="LOX/CH4",0.0,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.0,0.0)))))</f>
-        <v/>
-      </c>
-      <c r="H56" s="10">
-        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.0,IF(H21="LOX/LH2",0.0,IF(H21="LOX/CH4",0.0,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.0,0.0)))))</f>
-        <v/>
-      </c>
-      <c r="K56" s="10">
-        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.0,IF(K21="LOX/LH2",0.0,IF(K21="LOX/CH4",0.0,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.0,0.0)))))</f>
+      <c r="E56" s="21">
+        <f>IFERROR(E19*E43*1.15, "")</f>
+        <v/>
+      </c>
+      <c r="H56" s="21">
+        <f>IFERROR(H19*H43*1.15, "")</f>
+        <v/>
+      </c>
+      <c r="K56" s="21">
+        <f>IFERROR(K19*K43*1.15, "")</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="22" t="inlineStr">
-        <is>
-          <t>Residuals / Margin</t>
-        </is>
-      </c>
-      <c r="B57" s="12" t="inlineStr">
+      <c r="A57" s="23" t="inlineStr">
+        <is>
+          <t>TOTAL DRY MASS (Estimated)</t>
+        </is>
+      </c>
+      <c r="B57" s="24" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E57" s="10">
-        <f>IF(E22="","",E22/100*IF(E21="LOX/RP-1",0.5,IF(E21="LOX/LH2",0.8,IF(E21="LOX/CH4",0.5,IF(OR(E21="Solid HTPB",E21="Solid PBAN"),0.3,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="H57" s="10">
-        <f>IF(H22="","",H22/100*IF(H21="LOX/RP-1",0.5,IF(H21="LOX/LH2",0.8,IF(H21="LOX/CH4",0.5,IF(OR(H21="Solid HTPB",H21="Solid PBAN"),0.3,0.5)))))</f>
-        <v/>
-      </c>
-      <c r="K57" s="10">
-        <f>IF(K22="","",K22/100*IF(K21="LOX/RP-1",0.5,IF(K21="LOX/LH2",0.8,IF(K21="LOX/CH4",0.5,IF(OR(K21="Solid HTPB",K21="Solid PBAN"),0.3,0.5)))))</f>
+      <c r="E57" s="13">
+        <f>IFERROR(E46+E47+E48+E49+E50+E51+E52+E53+E54+E55+E56, "")</f>
+        <v/>
+      </c>
+      <c r="H57" s="13">
+        <f>IFERROR(H46+H47+H48+H49+H50+H51+H52+H53+H54+H55+H56, "")</f>
+        <v/>
+      </c>
+      <c r="K57" s="13">
+        <f>IFERROR(K46+K47+K48+K49+K50+K51+K52+K53+K54+K55+K56, "")</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="22" t="inlineStr">
-        <is>
-          <t>Engine System Total</t>
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>Dry Mass Override (enter known value)</t>
         </is>
       </c>
       <c r="B58" s="12" t="inlineStr">
@@ -1709,136 +1731,136 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="E58" s="21">
-        <f>IFERROR(E20*E45*1.15, "")</f>
-        <v/>
-      </c>
-      <c r="H58" s="21">
-        <f>IFERROR(H20*H45*1.15, "")</f>
-        <v/>
-      </c>
-      <c r="K58" s="21">
-        <f>IFERROR(K20*K45*1.15, "")</f>
-        <v/>
-      </c>
+      <c r="E58" s="10" t="n">
+        <v>22200</v>
+      </c>
+      <c r="H58" s="10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K58" s="10" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="23" t="inlineStr">
-        <is>
-          <t>TOTAL DRY MASS (Estimated)</t>
-        </is>
-      </c>
-      <c r="B59" s="24" t="inlineStr">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>Effective Dry Mass</t>
+        </is>
+      </c>
+      <c r="B59" s="12" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E59" s="13">
-        <f>IFERROR(E48+E49+E50+E51+E52+E53+E54+E55+E56+E57+E58, "")</f>
-        <v/>
-      </c>
-      <c r="H59" s="13">
-        <f>IFERROR(H48+H49+H50+H51+H52+H53+H54+H55+H56+H57+H58, "")</f>
-        <v/>
-      </c>
-      <c r="K59" s="13">
-        <f>IFERROR(K48+K49+K50+K51+K52+K53+K54+K55+K56+K57+K58, "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="8" t="inlineStr">
-        <is>
-          <t>Dry Mass Override (enter known value)</t>
-        </is>
-      </c>
-      <c r="B60" s="12" t="inlineStr">
+      <c r="E59" s="21">
+        <f>IF(E58&lt;&gt;"",E58,E57)</f>
+        <v/>
+      </c>
+      <c r="H59" s="21">
+        <f>IF(H58&lt;&gt;"",H58,H57)</f>
+        <v/>
+      </c>
+      <c r="K59" s="21">
+        <f>IF(K58&lt;&gt;"",K58,K57)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>PERFORMANCE CALCULATIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="25" t="inlineStr">
+        <is>
+          <t>MAX PAYLOAD TO ORBIT</t>
+        </is>
+      </c>
+      <c r="B62" s="26">
+        <f>IF(B14&gt;=3,IFERROR((K23-K25)/(EXP(K27/(K32*9.80665))-1)-(K59+K25)-B8, ""),IF(B14&gt;=2,IFERROR((H23-H25)/(EXP(H27/(H32*9.80665))-1)-(H59+H25)-B8, ""),IFERROR((E23-E25)/(EXP(E27/(E32*9.80665))-1)-(E59+E25)-B8, "")))</f>
+        <v/>
+      </c>
+      <c r="C62" s="27" t="inlineStr">
+        <is>
+          <t>← Solved from last stage: m_payload = (prop−rec)/(e^(ΔV/Isp·g₀)−1) − (dry+rec) − adapter  |  Recovery penalty: lower stage's actual ΔV drops (see verification); reduce that stage's ΔV fraction to propagate penalty to payload</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>GTO PERFORMANCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="25" t="inlineStr">
+        <is>
+          <t>MAX PAYLOAD TO GTO</t>
+        </is>
+      </c>
+      <c r="B65" s="26">
+        <f>IF(B14&gt;=3,IFERROR((K23-K25)/(EXP(K34/(K32*9.80665))-1)-(K59+K25)-B8, ""),IF(B14&gt;=2,IFERROR((H23-H25)/(EXP(H34/(H32*9.80665))-1)-(H59+H25)-B8, ""),IFERROR((E23-E25)/(EXP(E34/(E32*9.80665))-1)-(E59+E25)-B8, "")))</f>
+        <v/>
+      </c>
+      <c r="C65" s="27" t="inlineStr">
+        <is>
+          <t>← MIN across all stage constraints using GTO ΔV allocations: capacity_i = (prop−rec)/(e^(ΔV/Isp·g₀)−1) − (dry+rec) − gross_above − adapter</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>Gross Stage Mass (Prop + Dry)</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E60" s="10" t="n">
-        <v>22200</v>
-      </c>
-      <c r="H60" s="10" t="n">
-        <v>4000</v>
-      </c>
-      <c r="K60" s="10" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="8" t="inlineStr">
-        <is>
-          <t>Effective Dry Mass</t>
-        </is>
-      </c>
-      <c r="B61" s="12" t="inlineStr">
+      <c r="E66" s="21">
+        <f>IFERROR(E23+E59, "")</f>
+        <v/>
+      </c>
+      <c r="H66" s="21">
+        <f>IFERROR(H23+H59, "")</f>
+        <v/>
+      </c>
+      <c r="K66" s="21">
+        <f>IFERROR(K23+K59, "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>Burnout Mass m_f</t>
+        </is>
+      </c>
+      <c r="B67" s="12" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E61" s="21">
-        <f>IF(E60&lt;&gt;"",E60,E59)</f>
-        <v/>
-      </c>
-      <c r="H61" s="21">
-        <f>IF(H60&lt;&gt;"",H60,H59)</f>
-        <v/>
-      </c>
-      <c r="K61" s="21">
-        <f>IF(K60&lt;&gt;"",K60,K59)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="7" t="inlineStr">
-        <is>
-          <t>PERFORMANCE CALCULATIONS</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="25" t="inlineStr">
-        <is>
-          <t>MAX PAYLOAD TO ORBIT</t>
-        </is>
-      </c>
-      <c r="B64" s="26">
-        <f>IF(B15&gt;=3,IFERROR((K24-K26)/(EXP(K28/(K33*9.80665))-1)-(K61+K26)-B8, ""),IF(B15&gt;=2,IFERROR((H24-H26)/(EXP(H28/(H33*9.80665))-1)-(H61+H26)-B8, ""),IFERROR((E24-E26)/(EXP(E28/(E33*9.80665))-1)-(E61+E26)-B8, "")))</f>
-        <v/>
-      </c>
-      <c r="C64" s="27" t="inlineStr">
-        <is>
-          <t>← Solved from last stage: m_payload = (prop−rec)/(e^(ΔV/Isp·g₀)−1) − (dry+rec) − adapter  |  Recovery penalty: lower stage's actual ΔV drops (see verification); reduce that stage's ΔV fraction to propagate penalty to payload</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="18" customHeight="1">
-      <c r="A66" s="7" t="inlineStr">
-        <is>
-          <t>GTO PERFORMANCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="25" t="inlineStr">
-        <is>
-          <t>MAX PAYLOAD TO GTO</t>
-        </is>
-      </c>
-      <c r="B67" s="26">
-        <f>IF(B15&gt;=3,IFERROR((K24-K26)/(EXP(K35/(K33*9.80665))-1)-(K61+K26)-B8, ""),IF(B15&gt;=2,IFERROR((H24-H26)/(EXP(H35/(H33*9.80665))-1)-(H61+H26)-B8, ""),IFERROR((E24-E26)/(EXP(E35/(E33*9.80665))-1)-(E61+E26)-B8, "")))</f>
-        <v/>
-      </c>
-      <c r="C67" s="27" t="inlineStr">
-        <is>
-          <t>← MIN across all stage constraints using GTO ΔV allocations: capacity_i = (prop−rec)/(e^(ΔV/Isp·g₀)−1) − (dry+rec) − gross_above − adapter</t>
-        </is>
+      <c r="E67" s="21">
+        <f>IFERROR(E59+E25+IFERROR(H66*1,0)+IFERROR(K66*1,0)+B62+B8, "")</f>
+        <v/>
+      </c>
+      <c r="H67" s="21">
+        <f>IFERROR(H59+H25+IFERROR(K66*1,0)+B62+B8, "")</f>
+        <v/>
+      </c>
+      <c r="K67" s="21">
+        <f>IFERROR(K59+K25+B62+B8, "")</f>
+        <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>Gross Stage Mass (Prop + Dry)</t>
+          <t>Initial Mass m_0 (at ignition)</t>
         </is>
       </c>
       <c r="B68" s="12" t="inlineStr">
@@ -1847,70 +1869,70 @@
         </is>
       </c>
       <c r="E68" s="21">
-        <f>IFERROR(E24+E61, "")</f>
+        <f>IFERROR(E67+E23-E25, "")</f>
         <v/>
       </c>
       <c r="H68" s="21">
-        <f>IFERROR(H24+H61, "")</f>
+        <f>IFERROR(H67+H23-H25, "")</f>
         <v/>
       </c>
       <c r="K68" s="21">
-        <f>IFERROR(K24+K61, "")</f>
+        <f>IFERROR(K67+K23-K25, "")</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>Burnout Mass m_f</t>
+          <t>Mass Ratio (m₀ / m_f)</t>
         </is>
       </c>
       <c r="B69" s="12" t="inlineStr">
         <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E69" s="21">
-        <f>IFERROR(E61+E26+IFERROR(H68*1,0)+IFERROR(K68*1,0)+B64+B8, "")</f>
-        <v/>
-      </c>
-      <c r="H69" s="21">
-        <f>IFERROR(H61+H26+IFERROR(K68*1,0)+B64+B8, "")</f>
-        <v/>
-      </c>
-      <c r="K69" s="21">
-        <f>IFERROR(K61+K26+B64+B8, "")</f>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E69" s="28">
+        <f>IFERROR(E68/E67, "")</f>
+        <v/>
+      </c>
+      <c r="H69" s="28">
+        <f>IFERROR(H68/H67, "")</f>
+        <v/>
+      </c>
+      <c r="K69" s="28">
+        <f>IFERROR(K68/K67, "")</f>
         <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="8" t="inlineStr">
-        <is>
-          <t>Initial Mass m_0 (at ignition)</t>
-        </is>
-      </c>
-      <c r="B70" s="12" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E70" s="21">
-        <f>IFERROR(E69+E24-E26, "")</f>
-        <v/>
-      </c>
-      <c r="H70" s="21">
-        <f>IFERROR(H69+H24-H26, "")</f>
-        <v/>
-      </c>
-      <c r="K70" s="21">
-        <f>IFERROR(K69+K24-K26, "")</f>
+      <c r="A70" s="23" t="inlineStr">
+        <is>
+          <t>Actual Stage ΔV (verification)</t>
+        </is>
+      </c>
+      <c r="B70" s="24" t="inlineStr">
+        <is>
+          <t>m/s</t>
+        </is>
+      </c>
+      <c r="E70" s="13">
+        <f>IFERROR(E32*9.80665*LN(E69), "")</f>
+        <v/>
+      </c>
+      <c r="H70" s="13">
+        <f>IFERROR(H32*9.80665*LN(H69), "")</f>
+        <v/>
+      </c>
+      <c r="K70" s="13">
+        <f>IFERROR(K32*9.80665*LN(K69), "")</f>
         <v/>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>Mass Ratio (m₀ / m_f)</t>
+          <t>Thrust-to-Weight Ratio (at ignition)</t>
         </is>
       </c>
       <c r="B71" s="12" t="inlineStr">
@@ -1918,232 +1940,183 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E71" s="28">
-        <f>IFERROR(E70/E69, "")</f>
-        <v/>
-      </c>
-      <c r="H71" s="28">
-        <f>IFERROR(H70/H69, "")</f>
-        <v/>
-      </c>
-      <c r="K71" s="28">
-        <f>IFERROR(K70/K69, "")</f>
+      <c r="E71" s="29">
+        <f>IFERROR(E19*IFERROR(VLOOKUP(E18,'Engine DB'!$A:$K,7,0),0)*1000/(E68*9.80665), "")</f>
+        <v/>
+      </c>
+      <c r="H71" s="29">
+        <f>IFERROR(H19*IFERROR(VLOOKUP(H18,'Engine DB'!$A:$K,6,0),0)*1000/(H68*9.80665), "")</f>
+        <v/>
+      </c>
+      <c r="K71" s="29">
+        <f>IFERROR(K19*IFERROR(VLOOKUP(K18,'Engine DB'!$A:$K,6,0),0)*1000/(K68*9.80665), "")</f>
         <v/>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="23" t="inlineStr">
-        <is>
-          <t>Actual Stage ΔV (verification)</t>
-        </is>
-      </c>
-      <c r="B72" s="24" t="inlineStr">
+      <c r="A72" s="8" t="inlineStr">
+        <is>
+          <t>Propellant Mass Fraction</t>
+        </is>
+      </c>
+      <c r="B72" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E72" s="28">
+        <f>IFERROR(E23/E68, "")</f>
+        <v/>
+      </c>
+      <c r="H72" s="28">
+        <f>IFERROR(H23/H68, "")</f>
+        <v/>
+      </c>
+      <c r="K72" s="28">
+        <f>IFERROR(K23/K68, "")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>VEHICLE SUMMARY</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="30" t="inlineStr">
+        <is>
+          <t>Max Payload to LEO</t>
+        </is>
+      </c>
+      <c r="B75" s="31">
+        <f>B62</f>
+        <v/>
+      </c>
+      <c r="C75" s="32" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="30" t="inlineStr">
+        <is>
+          <t>Max Payload to GTO</t>
+        </is>
+      </c>
+      <c r="B76" s="31">
+        <f>B65</f>
+        <v/>
+      </c>
+      <c r="C76" s="32" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="33" t="inlineStr">
+        <is>
+          <t>LEO Payload Fraction (GLOW)</t>
+        </is>
+      </c>
+      <c r="B77" s="34">
+        <f>IFERROR(B62/E68*100, "")</f>
+        <v/>
+      </c>
+      <c r="C77" s="32" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="33" t="inlineStr">
+        <is>
+          <t>Total Vehicle ΔV (actual)</t>
+        </is>
+      </c>
+      <c r="B78" s="35">
+        <f>IFERROR(E70*1,0)+IFERROR(H70*1,0)+IFERROR(K70*1,0)</f>
+        <v/>
+      </c>
+      <c r="C78" s="32" t="inlineStr">
         <is>
           <t>m/s</t>
-        </is>
-      </c>
-      <c r="E72" s="13">
-        <f>IFERROR(E33*9.80665*LN(E71), "")</f>
-        <v/>
-      </c>
-      <c r="H72" s="13">
-        <f>IFERROR(H33*9.80665*LN(H71), "")</f>
-        <v/>
-      </c>
-      <c r="K72" s="13">
-        <f>IFERROR(K33*9.80665*LN(K71), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="8" t="inlineStr">
-        <is>
-          <t>Thrust-to-Weight Ratio (at ignition)</t>
-        </is>
-      </c>
-      <c r="B73" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E73" s="29">
-        <f>IFERROR(E20*IFERROR(VLOOKUP(E19,'Engine DB'!$A:$K,7,0),0)*1000/(E70*9.80665), "")</f>
-        <v/>
-      </c>
-      <c r="H73" s="29">
-        <f>IFERROR(H20*IFERROR(VLOOKUP(H19,'Engine DB'!$A:$K,6,0),0)*1000/(H70*9.80665), "")</f>
-        <v/>
-      </c>
-      <c r="K73" s="29">
-        <f>IFERROR(K20*IFERROR(VLOOKUP(K19,'Engine DB'!$A:$K,6,0),0)*1000/(K70*9.80665), "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
-          <t>Propellant Mass Fraction</t>
-        </is>
-      </c>
-      <c r="B74" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E74" s="28">
-        <f>IFERROR(E24/E70, "")</f>
-        <v/>
-      </c>
-      <c r="H74" s="28">
-        <f>IFERROR(H24/H70, "")</f>
-        <v/>
-      </c>
-      <c r="K74" s="28">
-        <f>IFERROR(K24/K70, "")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="7" t="inlineStr">
-        <is>
-          <t>VEHICLE SUMMARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="30" t="inlineStr">
-        <is>
-          <t>Max Payload to LEO</t>
-        </is>
-      </c>
-      <c r="B77" s="31">
-        <f>B64</f>
-        <v/>
-      </c>
-      <c r="C77" s="32" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="30" t="inlineStr">
-        <is>
-          <t>Max Payload to GTO</t>
-        </is>
-      </c>
-      <c r="B78" s="31">
-        <f>B67</f>
-        <v/>
-      </c>
-      <c r="C78" s="32" t="inlineStr">
-        <is>
-          <t>kg</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="33" t="inlineStr">
         <is>
-          <t>LEO Payload Fraction (GLOW)</t>
-        </is>
-      </c>
-      <c r="B79" s="34">
-        <f>IFERROR(B64/E70*100, "")</f>
+          <t>LEO ΔV Margin vs Mission</t>
+        </is>
+      </c>
+      <c r="B79" s="35">
+        <f>IFERROR(E70*1,0)+IFERROR(H70*1,0)+IFERROR(K70*1,0)-B40</f>
         <v/>
       </c>
       <c r="C79" s="32" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>m/s</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="33" t="inlineStr">
         <is>
-          <t>Total Vehicle ΔV (actual)</t>
+          <t>Gross Liftoff Mass (GLOW)</t>
         </is>
       </c>
       <c r="B80" s="35">
-        <f>IFERROR(E72*1,0)+IFERROR(H72*1,0)+IFERROR(K72*1,0)</f>
+        <f>IFERROR(E68, "")</f>
         <v/>
       </c>
       <c r="C80" s="32" t="inlineStr">
         <is>
-          <t>m/s</t>
+          <t>kg</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="33" t="inlineStr">
         <is>
-          <t>LEO ΔV Margin vs Mission</t>
+          <t>Total Propellant Mass</t>
         </is>
       </c>
       <c r="B81" s="35">
-        <f>IFERROR(E72*1,0)+IFERROR(H72*1,0)+IFERROR(K72*1,0)-B42</f>
+        <f>IFERROR(E23,0)+IFERROR(H23,0)+IFERROR(K23,0)</f>
         <v/>
       </c>
       <c r="C81" s="32" t="inlineStr">
         <is>
-          <t>m/s</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="33" t="inlineStr">
-        <is>
-          <t>Gross Liftoff Mass (GLOW)</t>
-        </is>
-      </c>
-      <c r="B82" s="35">
-        <f>IFERROR(E70, "")</f>
-        <v/>
-      </c>
-      <c r="C82" s="32" t="inlineStr">
-        <is>
           <t>kg</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="33" t="inlineStr">
-        <is>
-          <t>Total Propellant Mass</t>
-        </is>
-      </c>
-      <c r="B83" s="35">
-        <f>IFERROR(E24,0)+IFERROR(H24,0)+IFERROR(K24,0)</f>
-        <v/>
-      </c>
-      <c r="C83" s="32" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="22">
     <mergeCell ref="C8:L8"/>
-    <mergeCell ref="C67:L67"/>
+    <mergeCell ref="A64:K64"/>
+    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="A45:K45"/>
+    <mergeCell ref="A61:K61"/>
     <mergeCell ref="C13:L13"/>
-    <mergeCell ref="C15:L15"/>
-    <mergeCell ref="A66:K66"/>
-    <mergeCell ref="A37:K37"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="C62:L62"/>
+    <mergeCell ref="C42:L42"/>
     <mergeCell ref="G3:H3"/>
     <mergeCell ref="C14:L14"/>
+    <mergeCell ref="A74:K74"/>
     <mergeCell ref="A1:M1"/>
-    <mergeCell ref="C64:L64"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A47:K47"/>
-    <mergeCell ref="A76:K76"/>
+    <mergeCell ref="C65:L65"/>
     <mergeCell ref="C10:L10"/>
     <mergeCell ref="D3:E3"/>
-    <mergeCell ref="A17:K17"/>
-    <mergeCell ref="C44:L44"/>
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="C9:L9"/>
-    <mergeCell ref="A63:K63"/>
     <mergeCell ref="C12:L12"/>
     <mergeCell ref="A2:M2"/>
     <mergeCell ref="C11:L11"/>
@@ -2159,7 +2132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A99"/>
+  <dimension ref="A1:A120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2518,80 +2491,76 @@
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="36" t="inlineStr">
         <is>
-          <t>MAJOR SIMPLIFYING ASSUMPTIONS</t>
+          <t>SIMPLIFYING ASSUMPTIONS</t>
         </is>
       </c>
     </row>
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="37" t="inlineStr">
         <is>
-          <t>The following assumptions are baked into this model. Understanding them helps interpret results:</t>
+          <t>The model makes several simplifications. Some are standard engineering approximations; others are</t>
         </is>
       </c>
     </row>
     <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="37" t="inlineStr"/>
+      <c r="A58" s="37" t="inlineStr">
+        <is>
+          <t>ad hoc parameters added to bring outputs into agreement with known vehicles. Both kinds are listed</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="37" t="inlineStr">
         <is>
-          <t>1. GRAVITY LOSS MODEL</t>
+          <t>here so you know which numbers rest on physics and which require calibration.</t>
         </is>
       </c>
     </row>
     <row r="60" ht="16" customHeight="1">
-      <c r="A60" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Gravity loss = (Gravity Loss Coefficient / TWR_liftoff) + Recovery Trajectory Penalty.</t>
-        </is>
-      </c>
+      <c r="A60" s="37" t="inlineStr"/>
     </row>
     <row r="61" ht="16" customHeight="1">
-      <c r="A61" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   The TWR term captures the effect of liftoff acceleration on the gravity turn. The trajectory</t>
+      <c r="A61" s="36" t="inlineStr">
+        <is>
+          <t>── PHYSICS-BASED SIMPLIFICATIONS ─────────────────────────────────────────────────────────────────</t>
         </is>
       </c>
     </row>
     <row r="62" ht="16" customHeight="1">
-      <c r="A62" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   penalty is an additive correction for the extra gravity loss incurred by recovery-optimized</t>
-        </is>
-      </c>
+      <c r="A62" s="37" t="inlineStr"/>
     </row>
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   pitch profiles (shallower pitch angle = more time fighting gravity). Calibrate both inputs</t>
+          <t>1. EFFECTIVE ISP IS A LINEAR ATMOSPHERIC BLEND</t>
         </is>
       </c>
     </row>
     <row r="64" ht="16" customHeight="1">
       <c r="A64" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   against a known vehicle. Typical total gravity loss: Expendable ~1,200–1,500 m/s (penalty=0);</t>
+          <t xml:space="preserve">   Isp_eff = Isp_SL + Atm_Fraction × (Isp_vac - Isp_SL). The true relationship between ambient</t>
         </is>
       </c>
     </row>
     <row r="65" ht="16" customHeight="1">
       <c r="A65" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   ASDS ~1,700–2,000 m/s (penalty ~500 m/s); RTLS ~2,100–2,500 m/s (penalty ~900 m/s).</t>
+          <t xml:space="preserve">   pressure and nozzle exit pressure is a continuous altitude-integrated curve. The scalar Atm</t>
         </is>
       </c>
     </row>
     <row r="66" ht="16" customHeight="1">
       <c r="A66" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Remaining limitation: the model still cannot distinguish trajectory shape within a mission class</t>
+          <t xml:space="preserve">   Fraction input approximates the average. For a sea-level-optimized nozzle on a typical ascent</t>
         </is>
       </c>
     </row>
     <row r="67" ht="16" customHeight="1">
       <c r="A67" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   (e.g. a high-TWR expendable vs a low-TWR expendable will have the same penalty).</t>
+          <t xml:space="preserve">   profile this is a reasonable first-order approximation, but can be off by 5–10 s.</t>
         </is>
       </c>
     </row>
@@ -2601,197 +2570,328 @@
     <row r="69" ht="16" customHeight="1">
       <c r="A69" s="37" t="inlineStr">
         <is>
-          <t>2. EFFECTIVE ISP IS A LINEAR ATMOSPHERIC BLEND</t>
+          <t>2. RECOVERY IS MODELED AS A SINGLE BURN FROM DRY MASS</t>
         </is>
       </c>
     </row>
     <row r="70" ht="16" customHeight="1">
       <c r="A70" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Isp_eff = Isp_SL + Atm_Fraction × (Isp_vac - Isp_SL). The Atm Fraction input is a scalar</t>
+          <t xml:space="preserve">   Recovery Propellant = eff_dry × (e^(ΔV_rec / Isp / g₀) - 1). Real recovery sequences involve</t>
         </is>
       </c>
     </row>
     <row r="71" ht="16" customHeight="1">
       <c r="A71" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   approximation of what is actually a continuous altitude-pressure curve. For sea-level-optimized</t>
+          <t xml:space="preserve">   multiple discrete burns (entry burn from a partially-fueled stage, landing burn from near-dry),</t>
         </is>
       </c>
     </row>
     <row r="72" ht="16" customHeight="1">
       <c r="A72" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   nozzles this can be off by 5–10 s depending on the vehicle's ascent profile. Default: 0.6 for S1.</t>
+          <t xml:space="preserve">   each starting from a different initial mass. A single equivalent burn underestimates total</t>
         </is>
       </c>
     </row>
     <row r="73" ht="16" customHeight="1">
-      <c r="A73" s="37" t="inlineStr"/>
+      <c r="A73" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   recovery propellant somewhat — the error is typically small relative to total propellant.</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="16" customHeight="1">
-      <c r="A74" s="37" t="inlineStr">
-        <is>
-          <t>3. GLOW INCLUDES PAYLOAD (ITERATIVE — see note below)</t>
-        </is>
-      </c>
+      <c r="A74" s="37" t="inlineStr"/>
     </row>
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   GLOW includes the solved payload mass so TWR and gravity loss are self-consistent. This creates</t>
+          <t>3. FAIRING MASS IS NOT MODELED AS A JETTISON EVENT</t>
         </is>
       </c>
     </row>
     <row r="76" ht="16" customHeight="1">
       <c r="A76" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   a circular reference resolved by Excel's iterative calculation (File → Options → Formulas →</t>
+          <t xml:space="preserve">   A payload fairing (typically 1,700–2,000 kg for a 5m fairing) is jettisoned partway through S1</t>
         </is>
       </c>
     </row>
     <row r="77" ht="16" customHeight="1">
       <c r="A77" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Enable iterative calculation). The workbook is saved with iteration enabled. If you see a</t>
+          <t xml:space="preserve">   burn. The model does not treat this as a discrete staging event. Fairing mass can be added to the</t>
         </is>
       </c>
     </row>
     <row r="78" ht="16" customHeight="1">
       <c r="A78" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   circular reference error, ensure iterative calculation is turned on in your Excel settings.</t>
+          <t xml:space="preserve">   Payload Adapter Mass as a workaround, accepting that it is treated as dead weight all the way to</t>
         </is>
       </c>
     </row>
     <row r="79" ht="16" customHeight="1">
-      <c r="A79" s="37" t="inlineStr"/>
+      <c r="A79" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   orbit rather than being dropped mid-ascent.</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="16" customHeight="1">
-      <c r="A80" s="37" t="inlineStr">
-        <is>
-          <t>4. RECOVERY IS MODELED AS A SINGLE BURN FROM DRY MASS</t>
-        </is>
-      </c>
+      <c r="A80" s="37" t="inlineStr"/>
     </row>
     <row r="81" ht="16" customHeight="1">
       <c r="A81" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Recovery Propellant = eff_dry × (e^(ΔV_recovery / Isp / g₀) - 1). Real recovery sequences</t>
+          <t>4. ISP DOES NOT VARY WITH THROTTLE</t>
         </is>
       </c>
     </row>
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   have multiple burns (entry burn from partially-fueled stage, landing burn from near-dry stage),</t>
+          <t xml:space="preserve">   Engines are modeled at a fixed Isp regardless of throttle level. In reality, throttling shifts</t>
         </is>
       </c>
     </row>
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   each starting from different initial masses. A single-burn model slightly underestimates total</t>
+          <t xml:space="preserve">   chamber pressure and mixture ratio, changing Isp by ~1–3%. Effect on ascent performance is small.</t>
         </is>
       </c>
     </row>
     <row r="84" ht="16" customHeight="1">
-      <c r="A84" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   recovery propellant. The error is typically 5–15% of recovery propellant (~1–3% of total prop).</t>
-        </is>
-      </c>
+      <c r="A84" s="37" t="inlineStr"/>
     </row>
     <row r="85" ht="16" customHeight="1">
-      <c r="A85" s="37" t="inlineStr"/>
+      <c r="A85" s="37" t="inlineStr">
+        <is>
+          <t>5. GLOW EXCLUDES PAYLOAD (TWR IS SLIGHTLY OPTIMISTIC)</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="16" customHeight="1">
       <c r="A86" s="37" t="inlineStr">
         <is>
-          <t>5. FAIRING MASS IS NOT EXPLICITLY MODELED</t>
+          <t xml:space="preserve">   The liftoff TWR and gravity loss are computed from stage masses only — payload is not included in</t>
         </is>
       </c>
     </row>
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   The payload fairing (typically 1,700–2,000 kg for a 5m fairing) is jettisoned mid-ascent during</t>
+          <t xml:space="preserve">   GLOW. This makes TWR slightly higher and gravity loss slightly lower than the real vehicle.</t>
         </is>
       </c>
     </row>
     <row r="88" ht="16" customHeight="1">
       <c r="A88" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   S1 burn. This model does not account for fairing jettison as a discrete mass event. In practice,</t>
+          <t xml:space="preserve">   For typical payload fractions of 2–4% of GLOW the error is small but non-zero.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="16" customHeight="1">
-      <c r="A89" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   fairing mass is often included in the reported payload adapter mass as a workaround.</t>
-        </is>
-      </c>
+      <c r="A89" s="37" t="inlineStr"/>
     </row>
     <row r="90" ht="16" customHeight="1">
-      <c r="A90" s="37" t="inlineStr"/>
+      <c r="A90" s="36" t="inlineStr">
+        <is>
+          <t>── AD HOC CALIBRATION PARAMETERS ─────────────────────────────────────────────────────────────────</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="16" customHeight="1">
-      <c r="A91" s="37" t="inlineStr">
-        <is>
-          <t>6. GTO ΔV IS A FIXED INPUT</t>
-        </is>
-      </c>
+      <c r="A91" s="37" t="inlineStr"/>
     </row>
     <row r="92" ht="16" customHeight="1">
       <c r="A92" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   The GTO Orbital ΔV input (default 10,400 m/s) does not vary with launch site latitude, target</t>
+          <t>These inputs do not derive from first principles. They are curve-fit parameters — adjust them until</t>
         </is>
       </c>
     </row>
     <row r="93" ht="16" customHeight="1">
       <c r="A93" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   inclination, apogee altitude, or insertion strategy. GTO missions vary by 300–600 m/s depending</t>
+          <t>the model matches a vehicle you trust, then use that configuration for trades.</t>
         </is>
       </c>
     </row>
     <row r="94" ht="16" customHeight="1">
-      <c r="A94" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   on these parameters. Tune this value for specific mission comparisons.</t>
-        </is>
-      </c>
+      <c r="A94" s="37" t="inlineStr"/>
     </row>
     <row r="95" ht="16" customHeight="1">
-      <c r="A95" s="37" t="inlineStr"/>
+      <c r="A95" s="37" t="inlineStr">
+        <is>
+          <t>1. GRAVITY LOSS COEFFICIENT</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="16" customHeight="1">
       <c r="A96" s="37" t="inlineStr">
         <is>
-          <t>7. ISP DOES NOT VARY WITH THROTTLE</t>
+          <t xml:space="preserve">   Gravity loss = Coeff / TWR_liftoff. The 1/TWR relationship is a known trend, but the coefficient</t>
         </is>
       </c>
     </row>
     <row r="97" ht="16" customHeight="1">
       <c r="A97" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Engines are modeled at a fixed Isp. In reality, throttling changes chamber pressure and mixture</t>
+          <t xml:space="preserve">   value is empirical. Real gravity loss depends on the full pitch schedule integrated over the</t>
         </is>
       </c>
     </row>
     <row r="98" ht="16" customHeight="1">
       <c r="A98" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   ratio, shifting Isp by ~1–3%. This matters most for engines that throttle deeply (Merlin 1D</t>
+          <t xml:space="preserve">   entire ascent, not just liftoff TWR. The coefficient is adjusted until the total gravity loss</t>
         </is>
       </c>
     </row>
     <row r="99" ht="16" customHeight="1">
       <c r="A99" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   throttles to ~40% for landing burns). Effect on ascent performance is small but non-zero.</t>
+          <t xml:space="preserve">   produces the right mission ΔV for a reference vehicle. Default: 1,750.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="16" customHeight="1">
+      <c r="A100" s="37" t="inlineStr"/>
+    </row>
+    <row r="101" ht="16" customHeight="1">
+      <c r="A101" s="37" t="inlineStr">
+        <is>
+          <t>2. TRAJECTORY PENALTY</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="16" customHeight="1">
+      <c r="A102" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   An additive term on top of Coeff/TWR intended to capture extra gravity loss from a lofted or</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="16" customHeight="1">
+      <c r="A103" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   recovery-optimized ascent profile. The physical basis is real — recovery missions pitch</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="16" customHeight="1">
+      <c r="A104" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   differently to an expendable — but the magnitude is not derived from trajectory analysis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="16" customHeight="1">
+      <c r="A105" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   A single penalty is applied to both LEO and GTO mission ΔV. Whether the true penalty differs</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="16" customHeight="1">
+      <c r="A106" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   between mission types is unknown without trajectory simulation data, so we do not attempt to</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="16" customHeight="1">
+      <c r="A107" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   model them separately. Calibrate this value against a known LEO payload figure; accept that the</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="16" customHeight="1">
+      <c r="A108" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   same penalty will be applied to GTO and check that result against a known GTO figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="16" customHeight="1">
+      <c r="A109" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Default: 500 m/s (Falcon 9 ASDS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="16" customHeight="1">
+      <c r="A110" s="37" t="inlineStr"/>
+    </row>
+    <row r="111" ht="16" customHeight="1">
+      <c r="A111" s="37" t="inlineStr">
+        <is>
+          <t>3. GTO ORBITAL ΔV (FIXED INPUT)</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="16" customHeight="1">
+      <c r="A112" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   The total mission ΔV for a GTO mission is a fixed input (default 10,400 m/s). In reality this</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="16" customHeight="1">
+      <c r="A113" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   varies with launch site, target inclination, apogee altitude, and perigee insertion strategy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="16" customHeight="1">
+      <c r="A114" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Typical range is 10,000–10,800 m/s. Tune this to match a specific mission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="16" customHeight="1">
+      <c r="A115" s="37" t="inlineStr"/>
+    </row>
+    <row r="116" ht="16" customHeight="1">
+      <c r="A116" s="37" t="inlineStr">
+        <is>
+          <t>5. STAGE ΔV FRACTIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="16" customHeight="1">
+      <c r="A117" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   The LEO ΔV Fraction and GTO ΔV Fraction inputs split the total mission ΔV across stages.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="16" customHeight="1">
+      <c r="A118" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Optimal staging (Lagrange condition) gives a theoretical split, but real vehicles deviate from</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="16" customHeight="1">
+      <c r="A119" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   this due to recovery propellant, engine constraints, and trajectory shaping. These fractions are</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="16" customHeight="1">
+      <c r="A120" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   calibrated by iteration against known vehicles — they are not outputs of the model.</t>
         </is>
       </c>
     </row>

</xml_diff>